<commit_message>
Confirm Weigela Prism Magic Carpet and replace Delosperma with Calluna trio
</commit_message>
<xml_diff>
--- a/Oak_Lodge_Garden_Plant_Guide.xlsx
+++ b/Oak_Lodge_Garden_Plant_Guide.xlsx
@@ -4971,32 +4971,32 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>Delosperma 'Ice Cream Mix'</t>
+          <t>Calluna Trio Mix (3 plants)</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>Delosperma cooperi Ice Cream Series</t>
+          <t>Calluna vulgaris mixed cultivars</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Full sun; flowers open best in bright, warm conditions.</t>
+          <t>Full sun in an open position.</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>Drought-tolerant once established. Water sparingly and never leave the crown in wet winter soil.</t>
+          <t>Sprinkler supplied; keep the root zone moist while establishing but never waterlogged.</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>Sharp drainage is essential. Avoid rich feeding, trim away damaged growth in spring and protect from prolonged severe frost if the soil is wet.</t>
+          <t>Keep the soil acidic and free draining. Trim lightly after flowering, never back into bare old wood, and keep fallen leaves clear of the crowns.</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>A low evergreen succulent mat with mixed pink, orange and yellow daisy flowers from summer into autumn.</t>
+          <t>A three-plant mixed Calluna group with pink, white and lime-green flower-and-foliage interest from late summer into autumn.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add September houseplant records
</commit_message>
<xml_diff>
--- a/Oak_Lodge_Garden_Plant_Guide.xlsx
+++ b/Oak_Lodge_Garden_Plant_Guide.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plant Guide" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$G$162</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$G$164</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Plant Guide'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G162"/>
+  <dimension ref="A1:G164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6261,190 +6261,264 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Skimmia Pot</t>
+          <t>House · Sitting Room · ‘Gioia’ Fern</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Skimmia 'Cleopatra'</t>
+          <t>Bird’s Nest Fern ‘Gioia’</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
+          <t>Asplenium antiquum ‘Gioia’</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>Light to full shade, sheltered from harsh sun and drying wind.</t>
+          <t>Bright, indirect light; protect the fronds from direct sun through the glass.</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>Keep the shared compost consistently moist but well drained, preferably using rainwater.</t>
+          <t>Keep compost lightly moist but never saturated; water around the pot edge rather than into the centre rosette.</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>Mulch or top-dress with leaf mould or ericaceous compost. Prune only lightly after flowering and keep ivy stems away from its crown.</t>
+          <t>Give it steady warmth and higher humidity, removing only damaged fronds at the base.</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>Glossy evergreen foliage, fragrant ivory spring flowers and long-lasting red berries from autumn into winter.</t>
+          <t>Evergreen indoor foliage throughout the year; growth slows in lower winter light.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Skimmia Pot</t>
+          <t>House · Hallway · Staghorn Fern</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>Hedera helix 'Yellow Ripple'</t>
+          <t>Staghorn Fern</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>Hedera helix 'Golden Starlight' (Yellow Ripple)</t>
+          <t>Platycerium bifurcatum</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>Full shade to partial shade; shelter pale margins from scorching sun.</t>
+          <t>Bright, indirect light; avoid harsh midday sun and cold draughts.</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>Share the Skimmia's evenly moist, well-drained compost; check beneath the foliage before watering.</t>
+          <t>Check the growing medium before watering and let excess water drain completely; never keep the base wet.</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>Trim to keep the ivy within the pot and away from the Skimmia crown. Remove any all-green reverted shoots at their origin.</t>
+          <t>Maintain moderate humidity and keep the fern clear of direct radiator heat. Leave the brown papery shield fronds in place.</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>Evergreen lobed leaves with yellow-to-cream margins provide year-round trailing colour.</t>
+          <t>Evergreen antler-like fronds are the display throughout the year; growth is slower in winter.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Bed 2/3 Wall Pot</t>
+          <t>Skimmia Pot</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Viburnum 'Lisarose'</t>
+          <t>Skimmia 'Cleopatra'</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Viburnum tinus 'Lisarose'</t>
+          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>Sun, partial shade or shade, sheltered from cold drying winds.</t>
+          <t>Light to full shade, sheltered from harsh sun and drying wind.</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist while establishing; never leave the container waterlogged.</t>
+          <t>Keep the shared compost consistently moist but well drained, preferably using rainwater.</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>Use humus-rich, well-drained compost. Prune only after flowering if its size needs controlling.</t>
+          <t>Mulch or top-dress with leaf mould or ericaceous compost. Prune only lightly after flowering and keep ivy stems away from its crown.</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>Brick-red winter buds open to pink-and-white flowers, followed by dark blue ornamental berries.</t>
+          <t>Glossy evergreen foliage, fragrant ivory spring flowers and long-lasting red berries from autumn into winter.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Bed 2/3 Wall Pot</t>
+          <t>Skimmia Pot</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Vinca minor 'Illumination'</t>
+          <t>Hedera helix 'Yellow Ripple'</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Vinca minor 'Illumination'</t>
+          <t>Hedera helix 'Golden Starlight' (Yellow Ripple)</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>Sun to shade; foliage colours best in bright indirect light or partial shade.</t>
+          <t>Full shade to partial shade; shelter pale margins from scorching sun.</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>Moderate. Let the surface dry slightly without allowing the pot to dry completely.</t>
+          <t>Share the Skimmia's evenly moist, well-drained compost; check beneath the foliage before watering.</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>Trim trailing stems to shape and keep drainage holes clear. Do not plant into open ground without a spread plan.</t>
+          <t>Trim to keep the ivy within the pot and away from the Skimmia crown. Remove any all-green reverted shoots at their origin.</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>Golden evergreen foliage with narrow green margins and violet-blue flowers from spring into autumn.</t>
+          <t>Evergreen lobed leaves with yellow-to-cream margins provide year-round trailing colour.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
+          <t>Bed 2/3 Wall Pot</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Viburnum 'Lisarose'</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Viburnum tinus 'Lisarose'</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>Sun, partial shade or shade, sheltered from cold drying winds.</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>Keep evenly moist while establishing; never leave the container waterlogged.</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>Use humus-rich, well-drained compost. Prune only after flowering if its size needs controlling.</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>Brick-red winter buds open to pink-and-white flowers, followed by dark blue ornamental berries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>Bed 2/3 Wall Pot</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Vinca minor 'Illumination'</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Vinca minor 'Illumination'</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>Sun to shade; foliage colours best in bright indirect light or partial shade.</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>Moderate. Let the surface dry slightly without allowing the pot to dry completely.</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>Trim trailing stems to shape and keep drainage holes clear. Do not plant into open ground without a spread plan.</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>Golden evergreen foliage with narrow green margins and violet-blue flowers from spring into autumn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
           <t>Viburnum Pot</t>
         </is>
       </c>
-      <c r="B162" s="2" t="inlineStr">
+      <c r="B164" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus Spirit</t>
         </is>
       </c>
-      <c r="C162" s="2" t="inlineStr">
+      <c r="C164" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus 'Anvi' (Spirit)</t>
         </is>
       </c>
-      <c r="D162" s="2" t="inlineStr">
+      <c r="D164" s="2" t="inlineStr">
         <is>
           <t>Sun or partial shade, with shelter from cold drying winds.</t>
         </is>
       </c>
-      <c r="E162" s="2" t="inlineStr">
+      <c r="E164" s="2" t="inlineStr">
         <is>
           <t>Keep evenly moist but well drained while establishing; check the pot through dry and windy weather.</t>
         </is>
       </c>
-      <c r="F162" s="2" t="inlineStr">
+      <c r="F164" s="2" t="inlineStr">
         <is>
           <t>Prune only after flowering if needed. Refresh the top compost in spring and protect the container during prolonged severe cold.</t>
         </is>
       </c>
-      <c r="G162" s="2" t="inlineStr">
+      <c r="G164" s="2" t="inlineStr">
         <is>
           <t>Pink buds open to lightly fragrant creamy-white flowers from late winter into spring, followed by blue-black ornamental berries.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G162"/>
+  <autoFilter ref="A1:G164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Record September pots, hanging baskets and Front Bed 5 updates
</commit_message>
<xml_diff>
--- a/Oak_Lodge_Garden_Plant_Guide.xlsx
+++ b/Oak_Lodge_Garden_Plant_Guide.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plant Guide" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$G$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$G$170</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Plant Guide'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G164"/>
+  <dimension ref="A1:G170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3528,49 +3528,49 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Geranium</t>
+          <t>Helleborus Ice N' Roses Bennotta</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Pelargonium 'Trend Sophie Dark Red'</t>
+          <t>Helleborus × glandorfensis 'COSEH 6600'</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Partial shade to sun in a sheltered position.</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Moderate. Let compost dry slightly between waterings.</t>
+          <t>Keep compost evenly moist but freely drained; do not leave the crown waterlogged.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Deadhead regularly. Feed fortnightly. Not frost-hardy — overwinter indoors or treat as annual.</t>
+          <t>Remove tired leaves and faded flower stems in spring. Wear gloves when handling, and raise the pot so winter rain drains freely.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Dark red flower heads May–October; scented rounded leaves.</t>
+          <t>Deep pink to red outward-facing flowers from winter into spring above evergreen foliage.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Little Pot 1</t>
+          <t>Little Pot 2</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Petunia</t>
+          <t>Coreopsis Gold</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Petunia 'Vivini Blue Star'</t>
+          <t>Coreopsis 'Gold'</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -3580,91 +3580,91 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Regular; don't let compost dry out completely.</t>
+          <t>Moderate; the small pot dries quickly, but avoid permanently wet compost.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Deadhead spent blooms. Feed weekly. Tender annual.</t>
+          <t>Deadhead regularly for continuous flowering. Cut tired growth back by up to half for a second flush and keep the pot freely drained through winter.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Blue-white star-patterned flowers May–October.</t>
+          <t>Bright golden-yellow daisy flowers June–September above a compact leafy mound.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Little Pot 2</t>
+          <t>Cercis Pot</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Coreopsis Gold</t>
+          <t>Cercis 'Carolina Sweetheart'</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Coreopsis 'Gold'</t>
+          <t>Cercis canadensis 'Nccc1'</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Full sun in a warm position; shelter the pot from severe drying wind.</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Moderate; the small pot dries quickly, but avoid permanently wet compost.</t>
+          <t>Keep evenly moist while establishing. Water deeply when the upper compost starts to dry, without leaving the pot waterlogged.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Deadhead regularly for continuous flowering. Cut tired growth back by up to half for a second flush and keep the pot freely drained through winter.</t>
+          <t>Avoid routine pruning; remove only dead, damaged or crossing growth. Refresh the compost surface in spring and plan for a larger root run as the tree matures.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Bright golden-yellow daisy flowers June–September above a compact leafy mound.</t>
+          <t>Heart-shaped leaves open maroon-red and mature through green, cream and pink variegation; bare branches may carry pink-purple flowers in spring as the tree matures.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Cercis Pot</t>
+          <t>Front Pot</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Cercis 'Carolina Sweetheart'</t>
+          <t>Gazania 'Sunny Side Up'</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Cercis canadensis 'Nccc1'</t>
+          <t>Gazania rigens 'Sunny Side Up'</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Full sun in a warm position; shelter the pot from severe drying wind.</t>
+          <t>Full sun. Flowers close in shade and on overcast days.</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist while establishing. Water deeply when the upper compost starts to dry, without leaving the pot waterlogged.</t>
+          <t>Low to moderate. Drought-tolerant. Sharp drainage.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Avoid routine pruning; remove only dead, damaged or crossing growth. Refresh the compost surface in spring and plan for a larger root run as the tree matures.</t>
+          <t>Deadhead spent flowers to encourage more. Tender annual — replace each year. Does not recover from frost.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Heart-shaped leaves open maroon-red and mature through green, cream and pink variegation; bare branches may carry pink-purple flowers in spring as the tree matures.</t>
+          <t>Large cream-white daisy flowers with contrasting dark centres May–October; closes at night and on dull days.</t>
         </is>
       </c>
     </row>
@@ -3676,32 +3676,32 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Gazania 'Sunny Side Up'</t>
+          <t>Gazania 'Orange Flame'</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Gazania rigens 'Sunny Side Up'</t>
+          <t>Gazania rigens 'Orange Flame'</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Full sun. Flowers close in shade and on overcast days.</t>
+          <t>Full sun. Flowers close in shade.</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Low to moderate. Drought-tolerant. Sharp drainage.</t>
+          <t>Low to moderate. Drought-tolerant.</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Deadhead spent flowers to encourage more. Tender annual — replace each year. Does not recover from frost.</t>
+          <t>Deadhead to extend flowering. Tender annual — replace each year. Not frost-hardy.</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Large cream-white daisy flowers with contrasting dark centres May–October; closes at night and on dull days.</t>
+          <t>Vivid orange flame-patterned daisy flowers May–October; closes at night and on dull days.</t>
         </is>
       </c>
     </row>
@@ -3713,32 +3713,32 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Gazania 'Orange Flame'</t>
+          <t>Calibrachoa</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Gazania rigens 'Orange Flame'</t>
+          <t>Calibrachoa spp.</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Full sun. Flowers close in shade.</t>
+          <t>Full sun.</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Low to moderate. Drought-tolerant.</t>
+          <t>Keep evenly moist. Hates drying out.</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Deadhead to extend flowering. Tender annual — replace each year. Not frost-hardy.</t>
+          <t>Feed weekly with liquid tomato food. Self-cleaning — no deadheading needed. Tender annual.</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Vivid orange flame-patterned daisy flowers May–October; closes at night and on dull days.</t>
+          <t>Masses of small petunia-like flowers May–October. Continuous if fed.</t>
         </is>
       </c>
     </row>
@@ -3750,143 +3750,143 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Calibrachoa</t>
+          <t>Bacopa White</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Calibrachoa spp.</t>
+          <t>Sutera cordata (white cultivar)</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist. Hates drying out.</t>
+          <t>Keep evenly moist.</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Feed weekly with liquid tomato food. Self-cleaning — no deadheading needed. Tender annual.</t>
+          <t>Self-cleaning; no deadheading needed. Trim back if leggy. Tender annual.</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Masses of small petunia-like flowers May–October. Continuous if fed.</t>
+          <t>Tiny white flowers May–October; neat trailing habit.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Front Pot</t>
+          <t>Wall Pot 1</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Bacopa White</t>
+          <t>Phormium 'Flamingo'</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Sutera cordata (white cultivar)</t>
+          <t>Phormium 'Flamingo'</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Full sun for strongest foliage colour; shelter from severe cold wind.</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist.</t>
+          <t>Water while establishing, then let the upper compost dry slightly; never leave the pot waterlogged.</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Self-cleaning; no deadheading needed. Trim back if leggy. Tender annual.</t>
+          <t>Remove only damaged leaves at the base. Raise the pot for winter drainage and protect the crown during severe frost.</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Tiny white flowers May–October; neat trailing habit.</t>
+          <t>Evergreen, pink-striped sword-like leaves give year-round structure.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Wall Pot 1</t>
+          <t>Wall Pot 2</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Candy House Mix</t>
+          <t>Echinacea 'Mooodz Glory'</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Calibrachoa 'Candy House Mix'</t>
+          <t>Echinacea 'Hilmooglor'</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Full sun for strongest flowering; tolerates partial shade.</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Regular; do not let dry out. Water at the base.</t>
+          <t>Moderate. Water thoroughly, then let the upper compost begin to dry; never leave the crown in cold, wet compost.</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Feed weekly with liquid tomato food. Deadhead spent flowers. Tender annual — replace each season. Trim back if leggy to encourage bushy growth.</t>
+          <t>Deadhead fading flowers for further blooms, or retain selected cones for winter structure. Protect the pot from prolonged winter saturation.</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Prolific trailing flowers in mixed red, yellow and pink June–October; dies with first frost.</t>
+          <t>White, slightly drooping petals around golden-green cones from summer into autumn; dies back to a hardy crown in winter.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Wall Pot 2</t>
+          <t>Baskets</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Echinacea 'Mooodz Glory'</t>
+          <t>Trailing Fuchsia</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Echinacea 'Hilmooglor'</t>
+          <t>Fuchsia (trailing cultivar)</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Full sun for strongest flowering; tolerates partial shade.</t>
+          <t>Partial shade to full sun.</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Moderate. Water thoroughly, then let the upper compost begin to dry; never leave the crown in cold, wet compost.</t>
+          <t>Daily in hot weather; never let dry out completely.</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Deadhead fading flowers for further blooms, or retain selected cones for winter structure. Protect the pot from prolonged winter saturation.</t>
+          <t>Feed weekly. Deadhead spent flowers. Not frost-hardy — replace each year.</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>White, slightly drooping petals around golden-green cones from summer into autumn; dies back to a hardy crown in winter.</t>
+          <t>Pendant bicolour flowers June–October.</t>
         </is>
       </c>
     </row>
@@ -3898,32 +3898,32 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Trailing Fuchsia</t>
+          <t>Bacopa</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Fuchsia (trailing cultivar)</t>
+          <t>Sutera cordata</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Partial shade to full sun.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Daily in hot weather; never let dry out completely.</t>
+          <t>Keep evenly moist.</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Feed weekly. Deadhead spent flowers. Not frost-hardy — replace each year.</t>
+          <t>Self-cleaning; no deadheading needed. Trim back if leggy. Tender annual.</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Pendant bicolour flowers June–October.</t>
+          <t>Tiny white flowers May–October; neat trailing habit.</t>
         </is>
       </c>
     </row>
@@ -3935,12 +3935,12 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Bacopa</t>
+          <t>Trailing Lobelia</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Sutera cordata</t>
+          <t>Lobelia erinus (trailing)</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -3950,17 +3950,17 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist.</t>
+          <t>Keep moist; hates drying out.</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Self-cleaning; no deadheading needed. Trim back if leggy. Tender annual.</t>
+          <t>Trim back mid-season if it gets straggly. Tender annual.</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Tiny white flowers May–October; neat trailing habit.</t>
+          <t>Blue trailing flowers May–October.</t>
         </is>
       </c>
     </row>
@@ -3972,32 +3972,32 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Trailing Lobelia</t>
+          <t>Trailing Verbena</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Lobelia erinus (trailing)</t>
+          <t>Verbena (trailing cultivar)</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Full sun.</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Keep moist; hates drying out.</t>
+          <t>Regular; don't let dry out.</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Trim back mid-season if it gets straggly. Tender annual.</t>
+          <t>Deadhead to extend flowering. Tender annual.</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Blue trailing flowers May–October.</t>
+          <t>Clusters of flowers June–October.</t>
         </is>
       </c>
     </row>
@@ -4009,32 +4009,32 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Trailing Verbena</t>
+          <t>Petunia</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Verbena (trailing cultivar)</t>
+          <t>Petunia (cultivar unknown)</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Full sun to light partial shade.</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Regular; don't let dry out.</t>
+          <t>Check daily in warm weather; water thoroughly before the basket dries out.</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Deadhead to extend flowering. Tender annual.</t>
+          <t>Feed weekly during flowering and remove faded blooms and seed capsules. Trim bare stems back to leafy growth.</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Clusters of flowers June–October.</t>
+          <t>Funnel-shaped summer flowers from June until the first frost; cultivar unresolved.</t>
         </is>
       </c>
     </row>
@@ -4046,12 +4046,12 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Petunia</t>
+          <t>Calluna Trio Mix (2 plants)</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Petunia (cultivar unknown)</t>
+          <t>Calluna vulgaris mixed cultivars</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -4061,239 +4061,239 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Check daily in warm weather; water thoroughly before the basket dries out.</t>
+          <t>Keep compost lightly moist while establishing; never waterlog.</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Feed weekly during flowering and remove faded blooms and seed capsules. Trim bare stems back to leafy growth.</t>
+          <t>Use free-draining, preferably ericaceous compost. Trim lightly after flowering, never into bare wood.</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Funnel-shaped summer flowers from June until the first frost; cultivar unresolved.</t>
+          <t>Evergreen foliage and late-summer to autumn colour.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 1</t>
+          <t>Baskets</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Hydrangea</t>
+          <t>Viola 'Rocky Purple Picotee' (2 plants)</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Hydrangea macrophylla</t>
+          <t>Viola cornuta 'Rocky Purple Picotee'</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Morning sun, afternoon shade.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Thirsty — water well in dry spells.</t>
+          <t>Keep compost evenly moist, particularly in windy weather.</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Leave old flower heads over winter; prune to a strong bud in spring.</t>
+          <t>Deadhead faded flowers and seed pods to extend the display.</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Mophead flowers July–Sept; bare in winter.</t>
+          <t>Purple flowers with a pale picotee edge through the cool season.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 1</t>
+          <t>Baskets</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Lavender</t>
+          <t>Hedera helix 'Yellow Ripple' (2 plants)</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Lavandula angustifolia</t>
+          <t>Hedera helix 'Golden Starlight' (Yellow Ripple)</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Shade to sun; avoid prolonged scorching sun on pale foliage.</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Drought-tolerant.</t>
+          <t>Keep the shared basket compost evenly moist and well drained.</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Trim after flowering and again in spring; don't cut into old wood.</t>
+          <t>Trim trails to shape and keep stems clear of neighbouring crowns.</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Purple spikes June–Aug; aromatic year-round.</t>
+          <t>Evergreen variegated trails give structure through winter.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 2</t>
+          <t>Baskets</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'Inferno'</t>
+          <t>Pansy 'Fire' (2 plants)</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'Inferno'</t>
+          <t>Viola × wittrockiana 'Fire'</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; stronger light brings out the warm foliage colour.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Moderate while establishing. Avoid waterlogged soil.</t>
+          <t>Keep evenly moist but never saturated.</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Shelter from cold drying winds and protect in severe frost. Trim lightly in spring to keep a compact shape.</t>
+          <t>Remove faded flowers and seed pods regularly.</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Glossy green, cream, orange and red foliage intensifies in cooler weather; evergreen in a sheltered spot.</t>
+          <t>Cool-season flowers provide autumn-to-spring colour.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 2</t>
+          <t>Baskets</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'Pina Colada'</t>
+          <t>Pansy 'Rose Surprise' (2 plants)</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'Pina Colada'</t>
+          <t>Viola × wittrockiana 'Rose Surprise'</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; best colour in a bright, sheltered position.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Moderate while establishing. Let the soil drain between waterings.</t>
+          <t>Keep evenly moist but never saturated.</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Protect from severe frost and cold winds. Lightly trim any untidy growth in spring.</t>
+          <t>Remove faded flowers and seed pods regularly.</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Golden foliage develops orange and bronze tones through autumn and winter; evergreen when sheltered.</t>
+          <t>Cool-season flowers provide autumn-to-spring colour.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 2</t>
+          <t>Front Bed 1</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'City Knights'</t>
+          <t>Hydrangea</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'City Knights'</t>
+          <t>Hydrangea macrophylla</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; bright shelter gives the richest leaf colour.</t>
+          <t>Morning sun, afternoon shade.</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Moderate while establishing. Keep the root zone drained and do not allow prolonged drought in its first season.</t>
+          <t>Thirsty — water well in dry spells.</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Protect from severe frost and cold drying winds. Remove only damaged tips in spring and avoid forcing soft late growth with autumn feed.</t>
+          <t>Leave old flower heads over winter; prune to a strong bud in spring.</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Glossy evergreen foliage holds deep burgundy, red and dark green tones, strengthening the bed's winter colour.</t>
+          <t>Mophead flowers July–Sept; bare in winter.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 2</t>
+          <t>Front Bed 1</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Hebe 'Kiwi' (Horopito)</t>
+          <t>Lavender</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Hebe 'Kiwi'</t>
+          <t>Lavandula angustifolia</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a sheltered position.</t>
+          <t>Full sun.</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Moderate while establishing; avoid waterlogged winter soil.</t>
+          <t>Drought-tolerant.</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Deadhead faded spikes and trim lightly after flowering. Avoid cutting back into old bare wood.</t>
+          <t>Trim after flowering and again in spring; don't cut into old wood.</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Purple flower spikes in summer above glossy green leaves with dark new growth; evergreen.</t>
+          <t>Purple spikes June–Aug; aromatic year-round.</t>
         </is>
       </c>
     </row>
@@ -4305,180 +4305,180 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Polemonium 'Golden Feathers'</t>
+          <t>Coprosma 'Inferno'</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Polemonium 'Golden Feathers'</t>
+          <t>Coprosma 'Inferno'</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade; give afternoon shade in hot weather.</t>
+          <t>Full sun to partial shade; stronger light brings out the warm foliage colour.</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Moderate. Keep evenly moist but not waterlogged while establishing.</t>
+          <t>Moderate while establishing. Avoid waterlogged soil.</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>Deadhead after flowering and cut tired foliage back for fresh growth. Watch for powdery mildew in dry, crowded conditions.</t>
+          <t>Shelter from cold drying winds and protect in severe frost. Trim lightly in spring to keep a compact shape.</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>Gold-edged ferny foliage from spring; lilac-mauve bell flowers in spring and early summer; herbaceous in winter.</t>
+          <t>Glossy green, cream, orange and red foliage intensifies in cooler weather; evergreen in a sheltered spot.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 3</t>
+          <t>Front Bed 2</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Climbing Rose 'Super Fairy'</t>
+          <t>Coprosma 'Pina Colada'</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Rosa 'Helsufair'</t>
+          <t>Coprosma 'Pina Colada'</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Sun to light partial shade.</t>
+          <t>Full sun to partial shade; best colour in a bright, sheltered position.</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Deep water at the base in dry spells, especially while establishing.</t>
+          <t>Moderate while establishing. Let the soil drain between waterings.</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>Vigorous climber to about 2.5m high and 1.5m wide. Tie long shoots into the wall support and fan laterals out. Prune in late winter and deadhead after flowering.</t>
+          <t>Protect from severe frost and cold winds. Lightly trim any untidy growth in spring.</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Clusters of small, light-pink double flowers from June into autumn; deciduous in winter.</t>
+          <t>Golden foliage develops orange and bronze tones through autumn and winter; evergreen when sheltered.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 3</t>
+          <t>Front Bed 2</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Variegated Dogwood</t>
+          <t>Coprosma 'City Knights'</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Cornus alba 'Elegantissima'</t>
+          <t>Coprosma 'City Knights'</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Sun or partial shade; the leaf colour and winter stems are strongest in good light.</t>
+          <t>Full sun to partial shade; bright shelter gives the richest leaf colour.</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Moisture-loving. Water deeply while it re-establishes and during prolonged dry spells.</t>
+          <t>Moderate while establishing. Keep the root zone drained and do not allow prolonged drought in its first season.</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Mulch after planting. Once settled, remove about a third of the oldest stems at the base in March to encourage vivid new winter stems.</t>
+          <t>Protect from severe frost and cold drying winds. Remove only damaged tips in spring and avoid forcing soft late growth with autumn feed.</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>Cream-edged leaves spring–autumn; brilliant red stems provide the main display in winter.</t>
+          <t>Glossy evergreen foliage holds deep burgundy, red and dark green tones, strengthening the bed's winter colour.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 3</t>
+          <t>Front Bed 2</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Red Hot Poker</t>
+          <t>Hebe 'Kiwi' (Horopito)</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Kniphofia</t>
+          <t>Hebe 'Kiwi'</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Full sun for the strongest flowering.</t>
+          <t>Full sun to partial shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Moderate while re-establishing; drought-tolerant once rooted, but dislikes winter waterlogging.</t>
+          <t>Moderate while establishing; avoid waterlogged winter soil.</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>Keep the crown clear and well drained. Remove spent flower stems, tidy old foliage in spring and divide congested clumps every four or five years.</t>
+          <t>Deadhead faded spikes and trim lightly after flowering. Avoid cutting back into old bare wood.</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>Bold orange-red poker spikes July–September above strappy, mostly evergreen foliage.</t>
+          <t>Purple flower spikes in summer above glossy green leaves with dark new growth; evergreen.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 3</t>
+          <t>Front Bed 2</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Leucothoe 'Little Flames'</t>
+          <t>Polemonium 'Golden Feathers'</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Leucothoe 'Little Flames'</t>
+          <t>Polemonium 'Golden Feathers'</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; some shade helps the soil stay evenly moist.</t>
+          <t>Sun to partial shade; give afternoon shade in hot weather.</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Keep moist but well drained, especially while establishing. Use rainwater where practical.</t>
+          <t>Moderate. Keep evenly moist but not waterlogged while establishing.</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>Needs acidic soil. Mulch with leaf mould or composted bark and prune only to remove damaged growth or lightly reshape after flowering.</t>
+          <t>Deadhead after flowering and cut tired foliage back for fresh growth. Watch for powdery mildew in dry, crowded conditions.</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Evergreen leaves and stems flush vivid red when young, with clusters of small white urn-shaped flowers in spring.</t>
+          <t>Gold-edged ferny foliage from spring; lilac-mauve bell flowers in spring and early summer; herbaceous in winter.</t>
         </is>
       </c>
     </row>
@@ -4490,180 +4490,180 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Rose (pink)</t>
+          <t>Climbing Rose 'Super Fairy'</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Rosa — IDENTIFY</t>
+          <t>Rosa 'Helsufair'</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Sun.</t>
+          <t>Sun to light partial shade.</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Deep watering, mulch in spring.</t>
+          <t>Deep water at the base in dry spells, especially while establishing.</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>Prune late winter; deadhead through summer.</t>
+          <t>Vigorous climber to about 2.5m high and 1.5m wide. Tie long shoots into the wall support and fan laterals out. Prune in late winter and deadhead after flowering.</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>Flowers June–Sept; bare winter.</t>
+          <t>Clusters of small, light-pink double flowers from June into autumn; deciduous in winter.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 4</t>
+          <t>Front Bed 3</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>Photinia (existing canopy)</t>
+          <t>Variegated Dogwood</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Photinia (cultivar to confirm)</t>
+          <t>Cornus alba 'Elegantissima'</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Sun or partial shade; the leaf colour and winter stems are strongest in good light.</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>Water deeply only in prolonged dry periods once established.</t>
+          <t>Moisture-loving. Water deeply while it re-establishes and during prolonged dry spells.</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>Lightly prune after the spring flush if shaping is needed. Keep the new underplanting mulched and watered while it establishes around the existing roots.</t>
+          <t>Mulch after planting. Once settled, remove about a third of the oldest stems at the base in March to encourage vivid new winter stems.</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>Evergreen canopy; fresh growth is often bronze-red and white flower clusters can appear in spring.</t>
+          <t>Cream-edged leaves spring–autumn; brilliant red stems provide the main display in winter.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 4</t>
+          <t>Front Bed 3</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>The Pilgrim</t>
+          <t>Red Hot Poker</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Rosa 'Auswalker'</t>
+          <t>Kniphofia</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade. Aim for at least four hours of direct sun.</t>
+          <t>Full sun for the strongest flowering.</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>Deep water at the base during dry spells, especially while establishing.</t>
+          <t>Moderate while re-establishing; drought-tolerant once rooted, but dislikes winter waterlogging.</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>David Austin medium climber. Tie new canes into the support, fanning them horizontally where possible. Feed and mulch in spring; deadhead through summer; prune in late winter.</t>
+          <t>Keep the crown clear and well drained. Remove spent flower stems, tidy old foliage in spring and divide congested clumps every four or five years.</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>Soft yellow, rosette-shaped flowers with a tea fragrance from June into autumn; deciduous in winter.</t>
+          <t>Bold orange-red poker spikes July–September above strappy, mostly evergreen foliage.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 4</t>
+          <t>Front Bed 3</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>The Generous Gardener</t>
+          <t>Leucothoe 'Little Flames'</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>Rosa 'Ausdrawn'</t>
+          <t>Leucothoe 'Little Flames'</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade. Tolerates a little less sun than many climbing roses.</t>
+          <t>Full sun to partial shade; some shade helps the soil stay evenly moist.</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>Deep water at the base during dry spells, especially in its first two years.</t>
+          <t>Keep moist but well drained, especially while establishing. Use rainwater where practical.</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>David Austin medium climber. Train and tie in long shoots, feed and mulch in spring, deadhead repeat flowers and prune in late winter. Good disease resistance.</t>
+          <t>Needs acidic soil. Mulch with leaf mould or composted bark and prune only to remove damaged growth or lightly reshape after flowering.</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>Pale pink, cup-shaped flowers fading almost white, with a strong old-rose and musk fragrance; repeat flowers June–autumn.</t>
+          <t>Evergreen leaves and stems flush vivid red when young, with clusters of small white urn-shaped flowers in spring.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 4</t>
+          <t>Front Bed 3</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Physocarpus Cluster 1 (2 × Little Devil + 1 × Lady in Red)</t>
+          <t>Rose (pink)</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Physocarpus opulifolius 'Little Devil' &amp; 'Lady in Red'</t>
+          <t>Rosa — IDENTIFY</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade; foliage is darkest with good light.</t>
+          <t>Sun.</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>Sprinkler supplied. Check all three root balls through establishment and water deeply in dry spells.</t>
+          <t>Deep watering, mulch in spring.</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>Keep all three crowns distinct, with the taller Lady in Red rising through the two compact Little Devils. Renew individual shrubs from the base only when mature and congested.</t>
+          <t>Prune late winter; deadhead through summer.</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>Burgundy and red-bronze foliage spring to autumn with pale pink flower clusters in early summer; bare in winter.</t>
+          <t>Flowers June–Sept; bare winter.</t>
         </is>
       </c>
     </row>
@@ -4675,32 +4675,32 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>Physocarpus Cluster 2 (2 × Lady in Red + 1 × Little Devil)</t>
+          <t>Photinia (existing canopy)</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>Physocarpus opulifolius 'Lady in Red' &amp; 'Little Devil'</t>
+          <t>Photinia (cultivar to confirm)</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade; best foliage colour in brighter light.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>Sprinkler supplied. Check all three root balls through establishment and water deeply in dry spells.</t>
+          <t>Water deeply only in prolonged dry periods once established.</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>Keep the compact Little Devil readable against the two taller Lady in Reds. Remove a few oldest stems at the base only when congestion develops.</t>
+          <t>Lightly prune after the spring flush if shaping is needed. Keep the new underplanting mulched and watered while it establishes around the existing roots.</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>Red, bronze and burgundy foliage spring to autumn with pink flower clusters in summer; bare in winter.</t>
+          <t>Evergreen canopy; fresh growth is often bronze-red and white flower clusters can appear in spring.</t>
         </is>
       </c>
     </row>
@@ -4712,32 +4712,32 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Azalea japonica 'Silvester'</t>
+          <t>The Pilgrim</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Rhododendron 'Sylvester'</t>
+          <t>Rosa 'Auswalker'</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Partial or dappled shade in a sheltered position.</t>
+          <t>Full sun to light partial shade. Aim for at least four hours of direct sun.</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>Dropper supplied. Keep its shallow acidic root zone evenly moist, preferably with rainwater.</t>
+          <t>Deep water at the base during dry spells, especially while establishing.</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Grow shallowly in acidic, humus-rich soil and mulch with leaf mould. Deadhead carefully after flowering and prune only damaged or wayward growth.</t>
+          <t>David Austin medium climber. Tie new canes into the support, fanning them horizontally where possible. Feed and mulch in spring; deadhead through summer; prune in late winter.</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>Compact evergreen foliage with purple-pink flowers in late spring.</t>
+          <t>Soft yellow, rosette-shaped flowers with a tea fragrance from June into autumn; deciduous in winter.</t>
         </is>
       </c>
     </row>
@@ -4749,32 +4749,32 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>Nemesia 'Lady Penelope'</t>
+          <t>The Generous Gardener</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>Nemesia 'Lady Penelope' (best-fit identification)</t>
+          <t>Rosa 'Ausdrawn'</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade in a sheltered position.</t>
+          <t>Full sun to light partial shade. Tolerates a little less sun than many climbing roses.</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>Dropper supplied. Keep evenly moist while flowering but never waterlogged.</t>
+          <t>Deep water at the base during dry spells, especially in its first two years.</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>Trim tired flowering stems by about a third for another flush. Feed lightly while flowering and protect from frost.</t>
+          <t>David Austin medium climber. Train and tie in long shoots, feed and mulch in spring, deadhead repeat flowers and prune in late winter. Good disease resistance.</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>Fragrant rose-pink and white flowers with pink markings and a yellow eye from late spring into autumn.</t>
+          <t>Pale pink, cup-shaped flowers fading almost white, with a strong old-rose and musk fragrance; repeat flowers June–autumn.</t>
         </is>
       </c>
     </row>
@@ -4786,32 +4786,32 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Purple Gem</t>
+          <t>Physocarpus Cluster 1 (2 × Little Devil + 1 × Lady in Red)</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>Sarcococca hookeriana var. humilis 'Purple Gem'</t>
+          <t>Physocarpus opulifolius 'Little Devil' &amp; 'Lady in Red'</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Shade to partial shade.</t>
+          <t>Sun to partial shade; foliage is darkest with good light.</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>Water in dry spells while establishing; tolerates dry shade once settled.</t>
+          <t>Sprinkler supplied. Check all three root balls through establishment and water deeply in dry spells.</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>Evergreen winter-scented shrub. Keep ivy from engulfing it and prune only lightly after flowering if needed.</t>
+          <t>Keep all three crowns distinct, with the taller Lady in Red rising through the two compact Little Devils. Renew individual shrubs from the base only when mature and congested.</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>Glossy evergreen foliage and purple young stems; small fragrant winter flowers followed by dark berries.</t>
+          <t>Burgundy and red-bronze foliage spring to autumn with pale pink flower clusters in early summer; bare in winter.</t>
         </is>
       </c>
     </row>
@@ -4823,32 +4823,32 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>Rhododendron 'Libretto'</t>
+          <t>Physocarpus Cluster 2 (2 × Lady in Red + 1 × Little Devil)</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>Rhododendron 'Libretto'</t>
+          <t>Physocarpus opulifolius 'Lady in Red' &amp; 'Little Devil'</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>Light dappled shade, sheltered from cold drying wind and harsh early-morning sun.</t>
+          <t>Sun to partial shade; best foliage colour in brighter light.</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>Keep the shallow root zone evenly moist but never waterlogged. Prefer rainwater, especially in hard-water areas.</t>
+          <t>Sprinkler supplied. Check all three root balls through establishment and water deeply in dry spells.</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>Plant shallowly in acidic, humus-rich soil. Mulch with composted bark while keeping the stem clear; deadhead carefully and prune only dead or wayward growth after flowering.</t>
+          <t>Keep the compact Little Devil readable against the two taller Lady in Reds. Remove a few oldest stems at the base only when congestion develops.</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>Evergreen foliage all year; large dark-purple flowers with an olive-yellow flare in late May and early June.</t>
+          <t>Red, bronze and burgundy foliage spring to autumn with pink flower clusters in summer; bare in winter.</t>
         </is>
       </c>
     </row>
@@ -4860,32 +4860,32 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Festuca 'Elijah Blue' (3 plants)</t>
+          <t>Azalea japonica 'Silvester'</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>Festuca glauca 'Elijah Blue'</t>
+          <t>Rhododendron 'Sylvester'</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade.</t>
+          <t>Partial or dappled shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>Water regularly during the first season; drought tolerant once established.</t>
+          <t>Dropper supplied. Keep its shallow acidic root zone evenly moist, preferably with rainwater.</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>Comb out dead leaves in spring and divide congested clumps every few years. Do not routinely shear hard.</t>
+          <t>Grow shallowly in acidic, humus-rich soil and mulch with leaf mould. Deadhead carefully after flowering and prune only damaged or wayward growth.</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>Blue-grey, mostly evergreen foliage for year-round texture; airy flower stems in early summer.</t>
+          <t>Compact evergreen foliage with purple-pink flowers in late spring.</t>
         </is>
       </c>
     </row>
@@ -4897,32 +4897,32 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>Pieris 'Polar Passion'</t>
+          <t>Nemesia 'Lady Penelope'</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Pieris japonica 'Ppobas' (Polar Passion)</t>
+          <t>Nemesia 'Lady Penelope' (best-fit identification)</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Partial shade, sheltered from cold winds and harsh early sun.</t>
+          <t>Full sun to light partial shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist in acidic, well-drained soil; use rainwater where practical.</t>
+          <t>Dropper supplied. Keep evenly moist while flowering but never waterlogged.</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>Mulch with ericaceous material and remove only spent flowers or damaged stems. Do not apply lime.</t>
+          <t>Trim tired flowering stems by about a third for another flush. Feed lightly while flowering and protect from frost.</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>Colourful young foliage and hanging clusters of spring flowers above evergreen leaves.</t>
+          <t>Fragrant rose-pink and white flowers with pink markings and a yellow eye from late spring into autumn.</t>
         </is>
       </c>
     </row>
@@ -4934,32 +4934,32 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Dahlia 'Tampico'</t>
+          <t>Purple Gem</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>Dahlia Dalina Maxi Tampico ('Datretten')</t>
+          <t>Sarcococca hookeriana var. humilis 'Purple Gem'</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Full sun, sheltered from strong wind.</t>
+          <t>Shade to partial shade.</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>Water deeply whenever the upper soil begins to dry; do not leave the tuber in saturated ground.</t>
+          <t>Water in dry spells while establishing; tolerates dry shade once settled.</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>Deadhead to keep flowers coming and support stems if they begin to lean. Lift and store the tuber frost-free after the first frost, or protect it with a deep dry mulch in a mild winter.</t>
+          <t>Evergreen winter-scented shrub. Keep ivy from engulfing it and prune only lightly after flowering if needed.</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>Red-and-white decorative flowers from summer until frost; dormant tuber in winter.</t>
+          <t>Glossy evergreen foliage and purple young stems; small fragrant winter flowers followed by dark berries.</t>
         </is>
       </c>
     </row>
@@ -4971,32 +4971,32 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>Verbena 'Margaret's Memory'</t>
+          <t>Rhododendron 'Libretto'</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>Glandularia 'Margaret's Memory'</t>
+          <t>Rhododendron 'Libretto'</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade.</t>
+          <t>Light dappled shade, sheltered from cold drying wind and harsh early-morning sun.</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>Keep moist but well drained while establishing; avoid waterlogged winter soil.</t>
+          <t>Keep the shallow root zone evenly moist but never waterlogged. Prefer rainwater, especially in hard-water areas.</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>Deadhead or cut back after a flower flush. Take late-summer tip cuttings as insurance where winter cold or wet is severe.</t>
+          <t>Plant shallowly in acidic, humus-rich soil. Mulch with composted bark while keeping the stem clear; deadhead carefully and prune only dead or wayward growth after flowering.</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>Lilac-pink flowers with dark eyes from spring into late autumn; semi-evergreen in a sheltered winter.</t>
+          <t>Evergreen foliage all year; large dark-purple flowers with an olive-yellow flare in late May and early June.</t>
         </is>
       </c>
     </row>
@@ -5008,32 +5008,32 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Calluna Trio Mix (3 plants)</t>
+          <t>Festuca 'Elijah Blue' (3 plants)</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>Calluna vulgaris mixed cultivars</t>
+          <t>Festuca glauca 'Elijah Blue'</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>Full sun in an open position.</t>
+          <t>Full sun to light partial shade.</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>Sprinkler supplied; keep the root zone moist while establishing but never waterlogged.</t>
+          <t>Water regularly during the first season; drought tolerant once established.</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>Keep the soil acidic and free draining. Trim lightly after flowering, never back into bare old wood, and keep fallen leaves clear of the crowns.</t>
+          <t>Comb out dead leaves in spring and divide congested clumps every few years. Do not routinely shear hard.</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>A three-plant mixed Calluna group with pink, white and lime-green flower-and-foliage interest from late summer into autumn.</t>
+          <t>Blue-grey, mostly evergreen foliage for year-round texture; airy flower stems in early summer.</t>
         </is>
       </c>
     </row>
@@ -5045,32 +5045,32 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>Achillea</t>
+          <t>Pieris 'Polar Passion'</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>Achillea millefolium</t>
+          <t>Pieris japonica 'Ppobas' (Polar Passion)</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Partial shade, sheltered from cold winds and harsh early sun.</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>Low to moderate. Drought-tolerant once established.</t>
+          <t>Keep evenly moist in acidic, well-drained soil; use rainwater where practical.</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>Cut back after first flush for a second showing. Divide clumps every 2–3 years to keep vigorous. Good for cutting.</t>
+          <t>Mulch with ericaceous material and remove only spent flowers or damaged stems. Do not apply lime.</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>Flat-headed flower clusters in red, pink or yellow June–September; feathery aromatic foliage through the season.</t>
+          <t>Colourful young foliage and hanging clusters of spring flowers above evergreen leaves.</t>
         </is>
       </c>
     </row>
@@ -5082,180 +5082,180 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Azalea japonica 'Lotte'</t>
+          <t>Dahlia 'Tampico'</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>Rhododendron 'Lotte'</t>
+          <t>Dahlia Dalina Maxi Tampico ('Datretten')</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Partial or dappled shade in a sheltered position.</t>
+          <t>Full sun, sheltered from strong wind.</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>Dropper supplied. Keep its shallow acidic root zone evenly moist, preferably with rainwater.</t>
+          <t>Water deeply whenever the upper soil begins to dry; do not leave the tuber in saturated ground.</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>Grow shallowly in acidic, humus-rich soil and mulch with leaf mould. Deadhead carefully after flowering and prune only damaged growth.</t>
+          <t>Deadhead to keep flowers coming and support stems if they begin to lean. Lift and store the tuber frost-free after the first frost, or protect it with a deep dry mulch in a mild winter.</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>Compact glossy evergreen foliage with deep-pink flowers in late spring.</t>
+          <t>Red-and-white decorative flowers from summer until frost; dormant tuber in winter.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 5</t>
+          <t>Front Bed 4</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>Mexican Orange Blossom</t>
+          <t>Verbena 'Margaret's Memory'</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>Choisya ternata 'Sundance'</t>
+          <t>Glandularia 'Margaret's Memory'</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Sun for best colour.</t>
+          <t>Full sun to light partial shade.</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>Moderate.</t>
+          <t>Keep moist but well drained while establishing; avoid waterlogged winter soil.</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>Light prune after flowering to shape. Low-care.</t>
+          <t>Deadhead or cut back after a flower flush. Take late-summer tip cuttings as insurance where winter cold or wet is severe.</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>Golden evergreen foliage; scented white flowers spring &amp; again autumn.</t>
+          <t>Lilac-pink flowers with dark eyes from spring into late autumn; semi-evergreen in a sheltered winter.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 5</t>
+          <t>Front Bed 4</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Shrub Rose (cultivar to confirm)</t>
+          <t>Calluna Trio Mix (2 plants)</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>Rosa (Shrub Group; cultivar to confirm)</t>
+          <t>Calluna vulgaris mixed cultivars</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Full sun for the strongest flowering; tolerates light partial shade.</t>
+          <t>Full sun in an open position.</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>Water deeply in sustained dry spells, especially while flowering and forming hips.</t>
+          <t>Sprinkler supplied; keep the root zone moist while establishing but never waterlogged.</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>Remove dead, damaged and crossing stems in late winter. Thin congested growth and preserve sound hips where autumn colour and wildlife value are wanted.</t>
+          <t>Keep the soil acidic and free draining. Trim lightly after flowering, never back into bare old wood, and keep fallen leaves clear of the crowns.</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>Flowers are followed by red-orange rose hips — the fruits seen in the July photographs.</t>
+          <t>A two-plant mixed Calluna group with pink, white and lime-green flower-and-foliage interest from late summer into autumn.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 5</t>
+          <t>Front Bed 4</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>Bay Tree</t>
+          <t>Achillea</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>Laurus nobilis</t>
+          <t>Achillea millefolium</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a sheltered position.</t>
+          <t>Full sun.</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing and during prolonged drought; avoid waterlogged winter soil.</t>
+          <t>Low to moderate. Drought-tolerant once established.</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>Trim lightly in late spring or summer to retain the standard shape. Remove suckers and frost-damaged tips with secateurs.</t>
+          <t>Cut back after first flush for a second showing. Divide clumps every 2–3 years to keep vigorous. Good for cutting.</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>Aromatic evergreen leaves throughout the year; small spring flowers may be followed by dark berries on female plants.</t>
+          <t>Flat-headed flower clusters in red, pink or yellow June–September; feathery aromatic foliage through the season.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 5</t>
+          <t>Front Bed 4</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Japanese Skimmia</t>
+          <t>Azalea japonica 'Lotte'</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>Skimmia japonica (cultivar and sex to confirm)</t>
+          <t>Rhododendron 'Lotte'</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Partial shade to shade; shelter from the hottest afternoon sun.</t>
+          <t>Partial or dappled shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist but well drained, especially in dry summer weather.</t>
+          <t>Dropper supplied. Keep its shallow acidic root zone evenly moist, preferably with rainwater.</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>Mulch with leaf mould or ericaceous compost and prune only to remove damaged or awkward stems. Confirm sex and cultivar from flowers and fruit.</t>
+          <t>Grow shallowly in acidic, humus-rich soil and mulch with leaf mould. Deadhead carefully after flowering and prune only damaged growth.</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>Evergreen foliage and spring flower clusters; female or hermaphrodite forms can carry red berries when pollinated.</t>
+          <t>Compact glossy evergreen foliage with deep-pink flowers in late spring.</t>
         </is>
       </c>
     </row>
@@ -5267,32 +5267,32 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>Hardy Fuchsia (cultivar to confirm)</t>
+          <t>Mexican Orange Blossom</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>Fuchsia magellanica hybrid (cultivar to confirm)</t>
+          <t>Choisya ternata 'Sundance'</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade, sheltered from cold drying winds.</t>
+          <t>Sun for best colour.</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>Moist but well-drained soil; water in sustained dry spells while in flower.</t>
+          <t>Moderate.</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>Leave the top growth through winter, mulch the crown, then cut frost-damaged stems back to live buds in spring.</t>
+          <t>Light prune after flowering to shape. Low-care.</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>Pendant flowers from summer into autumn; top growth may die back in hard winters and regrow from the base.</t>
+          <t>Golden evergreen foliage; scented white flowers spring &amp; again autumn.</t>
         </is>
       </c>
     </row>
@@ -5304,32 +5304,32 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Clematis (cultivar to confirm)</t>
+          <t>Shrub Rose (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>Clematis viticella (cultivar to confirm)</t>
+          <t>Rosa (Shrub Group; cultivar to confirm)</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade, with a cool shaded root run.</t>
+          <t>Full sun for the strongest flowering; tolerates light partial shade.</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>Keep moist but well drained; soak the root zone during prolonged drought.</t>
+          <t>Water deeply in sustained dry spells, especially while flowering and forming hips.</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>Treat as pruning group 3 while the viticella identity remains the best fit: cut to strong buds 30–45cm above ground in late winter and tie in new shoots.</t>
+          <t>Remove dead, damaged and crossing stems in late winter. Thin congested growth and preserve sound hips where autumn colour and wildlife value are wanted.</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>Deciduous climber with abundant summer flowers on new growth.</t>
+          <t>Flowers are followed by red-orange rose hips — the fruits seen in the July photographs.</t>
         </is>
       </c>
     </row>
@@ -5341,32 +5341,32 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>Hydrangea 'Bloody Marie'</t>
+          <t>Bay Tree</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>Hydrangea paniculata 'Bloody Marie'</t>
+          <t>Laurus nobilis</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; afternoon shelter helps preserve moisture.</t>
+          <t>Full sun to partial shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>Keep the root zone consistently moist while establishing and through hot dry spells.</t>
+          <t>Water while establishing and during prolonged drought; avoid waterlogged winter soil.</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>Mulch in spring and prune in late winter or early spring before new growth, retaining a sound low framework. Panicle hydrangeas flower on the current season's shoots.</t>
+          <t>Trim lightly in late spring or summer to retain the standard shape. Remove suckers and frost-damaged tips with secateurs.</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>Large cream panicles age through pink toward red from July to September; deciduous in winter.</t>
+          <t>Aromatic evergreen leaves throughout the year; small spring flowers may be followed by dark berries on female plants.</t>
         </is>
       </c>
     </row>
@@ -5378,32 +5378,32 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Euphorbia 'Ascot Petite'</t>
+          <t>Japanese Skimmia</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>Euphorbia × martinii 'Ascot Petite'</t>
+          <t>Skimmia japonica (cultivar and sex to confirm)</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Full sun in a sheltered position.</t>
+          <t>Partial shade to shade; shelter from the hottest afternoon sun.</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing, then sparingly; sharp drainage is important in winter.</t>
+          <t>Keep evenly moist but well drained, especially in dry summer weather.</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>Remove old flowering stems at the base with gloves once replacement shoots are clear. Avoid disturbing the crown in cold wet weather.</t>
+          <t>Mulch with leaf mould or ericaceous compost and prune only to remove damaged or awkward stems. Confirm sex and cultivar from flowers and fruit.</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>Compact evergreen mound with yellow-green spring and early-summer flowerheads.</t>
+          <t>Evergreen foliage and spring flower clusters; female or hermaphrodite forms can carry red berries when pollinated.</t>
         </is>
       </c>
     </row>
@@ -5415,32 +5415,32 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>Flaming Silver</t>
+          <t>Hardy Fuchsia (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>Pieris japonica 'Flaming Silver'</t>
+          <t>Fuchsia magellanica hybrid (cultivar to confirm)</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>Partial shade to sun, sheltered from harsh morning frost.</t>
+          <t>Full sun to partial shade, sheltered from cold drying winds.</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist, especially in dry spells; do not let the rootball dry out.</t>
+          <t>Moist but well-drained soil; water in sustained dry spells while in flower.</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>Ericaceous shrub. Use rainwater where practical and mulch with ericaceous material; prune only lightly after flowering.</t>
+          <t>Leave the top growth through winter, mulch the crown, then cut frost-damaged stems back to live buds in spring.</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>Evergreen, cream-edged leaves with red spring growth and cream flowers in spring.</t>
+          <t>Pendant flowers from summer into autumn; top growth may die back in hard winters and regrow from the base.</t>
         </is>
       </c>
     </row>
@@ -5452,32 +5452,32 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Astrantia trio</t>
+          <t>Clematis (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>Astrantia major 'Buckland', 'Claret' &amp; 'Star of Love'</t>
+          <t>Clematis viticella (cultivar to confirm)</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>Sun to light shade.</t>
+          <t>Sun to partial shade, with a cool shaded root run.</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>Keep consistently moist during dry weather, particularly while re-establishing.</t>
+          <t>Keep moist but well drained; soak the root zone during prolonged drought.</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>Mulch annually with organic matter. Deadhead to prolong flowering and cut back tired stems after flowering.</t>
+          <t>Treat as pruning group 3 while the viticella identity remains the best fit: cut to strong buds 30–45cm above ground in late winter and tie in new shoots.</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>Pin-cushion flowers in blush, soft pink and claret shades through summer; foliage dies back in winter.</t>
+          <t>Deciduous climber with abundant summer flowers on new growth.</t>
         </is>
       </c>
     </row>
@@ -5489,32 +5489,32 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>Pittosporum 'Tom Thumb'</t>
+          <t>Hydrangea 'Bloody Marie'</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>Pittosporum tenuifolium 'Tom Thumb'</t>
+          <t>Hydrangea paniculata 'Bloody Marie'</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a sheltered position.</t>
+          <t>Full sun to partial shade; afternoon shelter helps preserve moisture.</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing; later only during prolonged drought. Avoid winter waterlogging.</t>
+          <t>Keep the root zone consistently moist while establishing and through hot dry spells.</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>Usually needs little pruning. Remove frost-damaged tips in late spring and protect from cold drying wind.</t>
+          <t>Mulch in spring and prune in late winter or early spring before new growth, retaining a sound low framework. Panicle hydrangeas flower on the current season's shoots.</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>Lime-green young leaves mature to deep purple, forming a dense rounded evergreen mound.</t>
+          <t>Large cream panicles age through pink toward red from July to September; deciduous in winter.</t>
         </is>
       </c>
     </row>
@@ -5526,32 +5526,32 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Gaura 'Gaudi Red'</t>
+          <t>Euphorbia 'Ascot Petite'</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>Oenothera lindheimeri 'Florgaured' (Gaudi Red)</t>
+          <t>Euphorbia × martinii 'Ascot Petite'</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Full sun in a warm, sheltered position.</t>
+          <t>Full sun in a sheltered position.</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing, then sparingly; sharp winter drainage is essential.</t>
+          <t>Water while establishing, then sparingly; sharp drainage is important in winter.</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>Deadhead for a longer display. Leave stems over winter and cut back after the worst frosts in spring.</t>
+          <t>Remove old flowering stems at the base with gloves once replacement shoots are clear. Avoid disturbing the crown in cold wet weather.</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>Deep pink-red flowers dance above burgundy-green foliage from summer into autumn.</t>
+          <t>Compact evergreen mound with yellow-green spring and early-summer flowerheads.</t>
         </is>
       </c>
     </row>
@@ -5563,32 +5563,32 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>Heather 'Bell's Extra Special'</t>
+          <t>Flaming Silver</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>Erica carnea 'Bell's Extra Special'</t>
+          <t>Pieris japonica 'Flaming Silver'</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade; stronger light keeps the foliage richly coloured.</t>
+          <t>Partial shade to sun, sheltered from harsh morning frost.</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing, then only in prolonged dry spells. Do not allow winter waterlogging.</t>
+          <t>Keep evenly moist, especially in dry spells; do not let the rootball dry out.</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>Grow in well-drained soil. Unlike Calluna, winter heath tolerates neutral to mildly alkaline conditions. Trim lightly after flowering without cutting into bare old wood.</t>
+          <t>Ericaceous shrub. Use rainwater where practical and mulch with ericaceous material; prune only lightly after flowering.</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>Golden evergreen foliage provides year-round colour, with small heath flowers in winter and early spring.</t>
+          <t>Evergreen, cream-edged leaves with red spring growth and cream flowers in spring.</t>
         </is>
       </c>
     </row>
@@ -5600,32 +5600,32 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Heather 'Tib'</t>
+          <t>Astrantia trio</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>Calluna vulgaris 'Tib'</t>
+          <t>Astrantia major 'Buckland', 'Claret' &amp; 'Star of Love'</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Full sun for compact growth and the best flower display.</t>
+          <t>Sun to light shade.</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing; afterwards it tolerates short dry spells but dislikes waterlogged soil.</t>
+          <t>Keep consistently moist during dry weather, particularly while re-establishing.</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>Needs acidic, well-drained soil. Clip the faded flower spikes lightly in early spring to keep the mound compact, never cutting into bare old wood.</t>
+          <t>Mulch annually with organic matter. Deadhead to prolong flowering and cut back tired stems after flowering.</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>Dark evergreen foliage carries double deep-pink flower spikes from July into early autumn.</t>
+          <t>Pin-cushion flowers in blush, soft pink and claret shades through summer; foliage dies back in winter.</t>
         </is>
       </c>
     </row>
@@ -5637,32 +5637,32 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>Bell Heather 'Providence' (2 plants)</t>
+          <t>Pittosporum 'Tom Thumb'</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>Daboecia cantabrica 'Providence'</t>
+          <t>Pittosporum tenuifolium 'Tom Thumb'</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a position sheltered from cold drying winds.</t>
+          <t>Full sun to partial shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist while establishing, using rainwater where practical; avoid both drought and waterlogging.</t>
+          <t>Water while establishing; later only during prolonged drought. Avoid winter waterlogging.</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>Grow in acidic, humus-rich but freely drained soil. Lightly trim faded stems after flowering without cutting into old wood.</t>
+          <t>Usually needs little pruning. Remove frost-damaged tips in late spring and protect from cold drying wind.</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>Evergreen mounds with comparatively large, deep rose-red bell flowers through summer and early autumn.</t>
+          <t>Lime-green young leaves mature to deep purple, forming a dense rounded evergreen mound.</t>
         </is>
       </c>
     </row>
@@ -5674,32 +5674,32 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Heather 'Leprechaun'</t>
+          <t>Gaura 'Gaudi Red'</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>Calluna vulgaris 'Leprechaun'</t>
+          <t>Oenothera lindheimeri 'Florgaured' (Gaudi Red)</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Full sun for the brightest foliage colour.</t>
+          <t>Full sun in a warm, sheltered position.</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing; later, water only during prolonged dry spells and keep the roots well drained.</t>
+          <t>Water while establishing, then sparingly; sharp winter drainage is essential.</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>Plant in acidic, freely drained soil. Clip faded flower spikes lightly in spring, avoiding cuts into bare old stems.</t>
+          <t>Deadhead for a longer display. Leave stems over winter and cut back after the worst frosts in spring.</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>A low evergreen mound with bright lime-gold foliage, pink-tinted new growth and small late-summer flowers.</t>
+          <t>Deep pink-red flowers dance above burgundy-green foliage from summer into autumn.</t>
         </is>
       </c>
     </row>
@@ -5711,32 +5711,32 @@
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>Heather 'Winter Chocolate'</t>
+          <t>Heather 'Bell's Extra Special'</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>Calluna vulgaris 'Winter Chocolate'</t>
+          <t>Erica carnea 'Bell's Extra Special'</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade; full sun produces the strongest foliage colour.</t>
+          <t>Full sun to light partial shade; stronger light keeps the foliage richly coloured.</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing; once rooted it tolerates short dry spells but must not sit wet.</t>
+          <t>Water while establishing, then only in prolonged dry spells. Do not allow winter waterlogging.</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>Grow in acidic, well-drained soil. Lightly remove old flower spikes in March to prevent the mound becoming woody and leggy.</t>
+          <t>Grow in well-drained soil. Unlike Calluna, winter heath tolerates neutral to mildly alkaline conditions. Trim lightly after flowering without cutting into bare old wood.</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>Golden foliage with pink tips in summer turns bronze and chocolate-red in winter; lavender flowers appear August–October.</t>
+          <t>Golden evergreen foliage provides year-round colour, with small heath flowers in winter and early spring.</t>
         </is>
       </c>
     </row>
@@ -5748,32 +5748,32 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Ceratostigma</t>
+          <t>Heather 'Tib'</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>Ceratostigma plumbaginoides</t>
+          <t>Calluna vulgaris 'Tib'</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; flowers and autumn colour are strongest in sun.</t>
+          <t>Full sun for compact growth and the best flower display.</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing, then only in prolonged drought. Prefers soil that drains freely.</t>
+          <t>Water while establishing; afterwards it tolerates short dry spells but dislikes waterlogged soil.</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>Allow room for the rhizomes to spread. Cut old top growth to the ground in spring once new shoots begin to show.</t>
+          <t>Needs acidic, well-drained soil. Clip the faded flower spikes lightly in early spring to keep the mound compact, never cutting into bare old wood.</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>Clear cobalt-blue flowers appear from late summer into autumn as the foliage develops vivid red tints; dormant in winter.</t>
+          <t>Dark evergreen foliage carries double deep-pink flower spikes from July into early autumn.</t>
         </is>
       </c>
     </row>
@@ -5785,32 +5785,32 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>Hypericum (cultivar to confirm)</t>
+          <t>Bell Heather 'Providence' (2 plants)</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>Hypericum (cultivar to confirm)</t>
+          <t>Daboecia cantabrica 'Providence'</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; more sun generally gives stronger flowering.</t>
+          <t>Full sun to partial shade in a position sheltered from cold drying winds.</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing, then during prolonged dry spells only. Avoid persistently waterlogged soil.</t>
+          <t>Keep evenly moist while establishing, using rainwater where practical; avoid both drought and waterlogging.</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>Trim lightly in early spring and remove any weak or damaged stems. Confirm the cultivar from its label, flowers and berries before cultivar-specific pruning.</t>
+          <t>Grow in acidic, humus-rich but freely drained soil. Lightly trim faded stems after flowering without cutting into old wood.</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>A compact shrub grown for golden flowers with prominent stamens and, depending on cultivar, colourful ornamental berries.</t>
+          <t>Evergreen mounds with comparatively large, deep rose-red bell flowers through summer and early autumn.</t>
         </is>
       </c>
     </row>
@@ -5822,32 +5822,32 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Bluebell Creeper</t>
+          <t>Heather 'Leprechaun'</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>Billardiera heterophylla (syn. Sollya heterophylla)</t>
+          <t>Calluna vulgaris 'Leprechaun'</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a warm, sheltered position.</t>
+          <t>Full sun for the brightest foliage colour.</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist while establishing, then water during dry spells; avoid waterlogged winter soil.</t>
+          <t>Water while establishing; later, water only during prolonged dry spells and keep the roots well drained.</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>Tie new shoots into support and trim after flowering to control the twining growth. Protect the root area and young stems during hard frost.</t>
+          <t>Plant in acidic, freely drained soil. Clip faded flower spikes lightly in spring, avoiding cuts into bare old stems.</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>A slender evergreen climber with nodding blue bell flowers from summer into autumn, followed by narrow berries when pollinated.</t>
+          <t>A low evergreen mound with bright lime-gold foliage, pink-tinted new growth and small late-summer flowers.</t>
         </is>
       </c>
     </row>
@@ -5859,32 +5859,32 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>Hebe 'Rhubarb and Custard'</t>
+          <t>Heather 'Winter Chocolate'</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Veronica 'Tull 302' (Rhubarb and Custard)</t>
+          <t>Calluna vulgaris 'Winter Chocolate'</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a warm, sheltered spot.</t>
+          <t>Full sun to light partial shade; full sun produces the strongest foliage colour.</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>Moderate while establishing; drought-tolerant later, but avoid winter waterlogging.</t>
+          <t>Water while establishing; once rooted it tolerates short dry spells but must not sit wet.</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>Lightly trim after flowering to keep its rounded shape and protect from severe frost or cold drying winds.</t>
+          <t>Grow in acidic, well-drained soil. Lightly remove old flower spikes in March to prevent the mound becoming woody and leggy.</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>Cream-edged grey-green leaves flush pink and rhubarb-red in cold weather; short purple flower spikes appear in mid- to late summer.</t>
+          <t>Golden foliage with pink tips in summer turns bronze and chocolate-red in winter; lavender flowers appear August–October.</t>
         </is>
       </c>
     </row>
@@ -5896,32 +5896,32 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Salvia 'Salgoon Lake Blueberry'</t>
+          <t>Viola 'Rocky Purple Picotee'</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Salvia 'Tl1016' (Salgoon Lake Blueberry)</t>
+          <t>Viola cornuta 'Rocky Purple Picotee'</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>Full sun in a warm, sheltered position.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>Water regularly while establishing; once rooted it has good heat and drought tolerance, provided drainage is sharp.</t>
+          <t>Keep evenly moist while establishing; do not allow the planting pocket to become waterlogged.</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>Deadhead to prolong flowering. Leave top growth over winter, mulch the crown and cut back after the worst frosts in spring; take cuttings as insurance in colder winters.</t>
+          <t>Deadhead faded flowers and seed pods regularly to prolong the cool-season display.</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>Compact upright growth to around 60cm with rich blueberry-purple flowers and near-black calyces from summer into autumn.</t>
+          <t>Purple flowers with pale picotee margins through autumn, winter and spring.</t>
         </is>
       </c>
     </row>
@@ -5933,592 +5933,814 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>Fern 'Jurassic Gold'</t>
+          <t>Ceratostigma</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Dryopteris wallichiana 'Hollasic' (Jurassic Gold)</t>
+          <t>Ceratostigma plumbaginoides</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>Full shade in a sheltered position.</t>
+          <t>Full sun to partial shade; flowers and autumn colour are strongest in sun.</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>Shares the existing sprinkler with location 10. Keep moist but well drained while establishing.</t>
+          <t>Water while establishing, then only in prolonged drought. Prefers soil that drains freely.</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>Mulch well over moist soil, keeping the crown clear. Remove dead or damaged fronds as needed and protect new croziers from late frost and slugs.</t>
+          <t>Allow room for the rhizomes to spread. Cut old top growth to the ground in spring once new shoots begin to show.</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>Rose-tinted young fronds mature through bright gold to green; deciduous to semi-evergreen depending on winter.</t>
+          <t>Clear cobalt-blue flowers appear from late summer into autumn as the foliage develops vivid red tints; dormant in winter.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Front Stone Trough</t>
+          <t>Front Bed 5</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Hosta</t>
+          <t>Hypericum (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Hosta</t>
+          <t>Hypericum (cultivar to confirm)</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>Part to full shade.</t>
+          <t>Full sun to partial shade; more sun generally gives stronger flowering.</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>Keep moist; never bone-dry in the trough.</t>
+          <t>Water while establishing, then during prolonged dry spells only. Avoid persistently waterlogged soil.</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>Watch for slugs/snails. Divide clumps in spring.</t>
+          <t>Trim lightly in early spring and remove any weak or damaged stems. Confirm the cultivar from its label, flowers and berries before cultivar-specific pruning.</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>Fresh leaves spring; dies back over winter.</t>
+          <t>A compact shrub grown for golden flowers with prominent stamens and, depending on cultivar, colourful ornamental berries.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Front Box Hedge</t>
+          <t>Front Bed 5</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>Wall Cotoneaster (species to confirm)</t>
+          <t>Bluebell Creeper</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Cotoneaster (species to confirm)</t>
+          <t>Billardiera heterophylla (syn. Sollya heterophylla)</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>Sun to part shade.</t>
+          <t>Full sun to partial shade in a warm, sheltered position.</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing; once settled, water only in prolonged dry spells.</t>
+          <t>Keep evenly moist while establishing, then water during dry spells; avoid waterlogged winter soil.</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>Train or lightly prune after flowering to keep growth clear of paths and masonry. Do not use box-blight or box-caterpillar treatments. Confirm the species from flowers, berries and leaf undersides.</t>
+          <t>Tie new shoots into support and trim after flowering to control the twining growth. Protect the root area and young stems during hard frost.</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>Small leaves on herringbone stems; flowers in late spring or summer followed by red berries. Evergreen or semi-evergreen depending on species and winter.</t>
+          <t>A slender evergreen climber with nodding blue bell flowers from summer into autumn, followed by narrow berries when pollinated.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Front Pots</t>
+          <t>Front Bed 5</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Mixed Pot</t>
+          <t>Hebe 'Rhubarb and Custard'</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>Mixed seasonal planting — contents to confirm</t>
+          <t>Veronica 'Tull 302' (Rhubarb and Custard)</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>Bright outdoor position; confirm the needs of each constituent plant when identified.</t>
+          <t>Full sun to partial shade in a warm, sheltered spot.</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>Check the compost frequently in warm or windy weather; supplied by an adjustable sprinkler.</t>
+          <t>Moderate while establishing; drought-tolerant later, but avoid winter waterlogging.</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>Deadhead finished flowers, keep the drainage holes clear and record the individual plants and cultivars as labels or clearer photographs become available.</t>
+          <t>Lightly trim after flowering to keep its rounded shape and protect from severe frost or cold drying winds.</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>A mixed seasonal container providing varied flower colour; exact contents remain unresolved.</t>
+          <t>Cream-edged grey-green leaves flush pink and rhubarb-red in cold weather; short purple flower spikes appear in mid- to late summer.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Front Pots</t>
+          <t>Front Bed 5</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>Fuchsia Pot</t>
+          <t>Salvia 'Salgoon Lake Blueberry'</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Fuchsia cultivars — identities to confirm</t>
+          <t>Salvia 'Tl1016' (Salgoon Lake Blueberry)</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>Bright light or partial shade, protected from the harshest reflected afternoon heat.</t>
+          <t>Full sun in a warm, sheltered position.</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>Keep the compost evenly moist but freely drained; supplied by an adjustable sprinkler.</t>
+          <t>Water regularly while establishing; once rooted it has good heat and drought tolerance, provided drainage is sharp.</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>Deadhead for continued flowering, check the sprinkler reaches the compost rather than only the foliage, and confirm whether the plants are hardy before winter.</t>
+          <t>Deadhead to prolong flowering. Leave top growth over winter, mulch the crown and cut back after the worst frosts in spring; take cuttings as insurance in colder winters.</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>Pendant Fuchsia flowers through summer and autumn; exact cultivars and winter hardiness remain unresolved.</t>
+          <t>Compact upright growth to around 60cm with rich blueberry-purple flowers and near-black calyces from summer into autumn.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Front Fruit Trees</t>
+          <t>Front Bed 5</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Apple Tree</t>
+          <t>Fern 'Jurassic Gold'</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>Malus domestica</t>
+          <t>Dryopteris wallichiana 'Hollasic' (Jurassic Gold)</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Full shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>Water well in dry spells while fruiting.</t>
+          <t>Shares the existing sprinkler with location 10. Keep moist but well drained while establishing.</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>Winter prune for shape and airflow; thin fruit in June if heavy.</t>
+          <t>Mulch well over moist soil, keeping the crown clear. Remove dead or damaged fronds as needed and protect new croziers from late frost and slugs.</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>Blossom April–May; fruit late summer–autumn.</t>
+          <t>Rose-tinted young fronds mature through bright gold to green; deciduous to semi-evergreen depending on winter.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Front Fruit Trees</t>
+          <t>Front Stone Trough</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>Damson Tree</t>
+          <t>Hosta</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>Prunus domestica subsp. insititia (cultivar to confirm)</t>
+          <t>Hosta</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>Full sun for reliable blossom and fruit ripening.</t>
+          <t>Part to full shade.</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>Water deeply during prolonged dry spells, especially from fruit set to harvest.</t>
+          <t>Keep moist; never bone-dry in the trough.</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>Prune only in dry summer weather to reduce silver-leaf and canker risk; remove suckers from below the graft.</t>
+          <t>Watch for slugs/snails. Divide clumps in spring.</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>White spring blossom followed by blue-black damsons in late summer or early autumn.</t>
+          <t>Fresh leaves spring; dies back over winter.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Front Gate Tree</t>
+          <t>Front Box Hedge</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>Weeping Crab Apple (cultivar to confirm)</t>
+          <t>Wall Cotoneaster (species to confirm)</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>Malus (weeping cultivar; 'Red Jade' is a best-fit possibility)</t>
+          <t>Cotoneaster (species to confirm)</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>Full sun for the best blossom, fruit colour and balanced growth.</t>
+          <t>Sun to part shade.</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>Water deeply during prolonged drought, particularly while establishing and while fruit is swelling.</t>
+          <t>Water while establishing; once settled, water only in prolonged dry spells.</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>Remove dead, damaged and crossing wood in winter, preserving the natural weeping framework. Record blossom and ripe-fruit details before naming the cultivar.</t>
+          <t>Train or lightly prune after flowering to keep growth clear of paths and masonry. Do not use box-blight or box-caterpillar treatments. Confirm the species from flowers, berries and leaf undersides.</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>Spring blossom followed by small ornamental crab apples that can persist into autumn and winter.</t>
+          <t>Small leaves on herringbone stems; flowers in late spring or summer followed by red berries. Evergreen or semi-evergreen depending on species and winter.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>House · Hallway · Kentia Palm</t>
+          <t>Front Pots</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>Kentia Palm — assumed</t>
+          <t>Mixed Pot</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>Howea forsteriana</t>
+          <t>Mixed seasonal planting — contents to confirm</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>Bright indirect light; protect the fronds from strong direct sun.</t>
+          <t>Bright outdoor position; confirm the needs of each constituent plant when identified.</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>Check the upper few centimetres of compost before watering, then drain fully and empty the white cachepot.</t>
+          <t>Check the compost frequently in warm or windy weather; supplied by an adjustable sprinkler.</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>Maintain moderate humidity, keep away from cold draughts and radiators, and feed monthly during active spring and summer growth.</t>
+          <t>Deadhead finished flowers, keep the drainage holes clear and record the individual plants and cultivars as labels or clearer photographs become available.</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>Evergreen indoor foliage throughout the year; growth slows as light levels fall in winter.</t>
+          <t>A mixed seasonal container providing varied flower colour; exact contents remain unresolved.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>House · Sitting Room · ‘Gioia’ Fern</t>
+          <t>Front Pots</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Bird’s Nest Fern ‘Gioia’</t>
+          <t>Fuchsia Pot</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>Asplenium antiquum ‘Gioia’</t>
+          <t>Fuchsia cultivars — identities to confirm</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>Bright, indirect light; protect the fronds from direct sun through the glass.</t>
+          <t>Bright light or partial shade, protected from the harshest reflected afternoon heat.</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>Keep compost lightly moist but never saturated; water around the pot edge rather than into the centre rosette.</t>
+          <t>Keep the compost evenly moist but freely drained; supplied by an adjustable sprinkler.</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>Give it steady warmth and higher humidity, removing only damaged fronds at the base.</t>
+          <t>Deadhead for continued flowering, check the sprinkler reaches the compost rather than only the foliage, and confirm whether the plants are hardy before winter.</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>Evergreen indoor foliage throughout the year; growth slows in lower winter light.</t>
+          <t>Pendant Fuchsia flowers through summer and autumn; exact cultivars and winter hardiness remain unresolved.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>House · Hallway · Staghorn Fern</t>
+          <t>Front Fruit Trees</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>Staghorn Fern</t>
+          <t>Apple Tree</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>Platycerium bifurcatum</t>
+          <t>Malus domestica</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>Bright, indirect light; avoid harsh midday sun and cold draughts.</t>
+          <t>Full sun.</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>Check the growing medium before watering and let excess water drain completely; never keep the base wet.</t>
+          <t>Water well in dry spells while fruiting.</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>Maintain moderate humidity and keep the fern clear of direct radiator heat. Leave the brown papery shield fronds in place.</t>
+          <t>Winter prune for shape and airflow; thin fruit in June if heavy.</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>Evergreen antler-like fronds are the display throughout the year; growth is slower in winter.</t>
+          <t>Blossom April–May; fruit late summer–autumn.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Skimmia Pot</t>
+          <t>Front Fruit Trees</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Skimmia 'Cleopatra'</t>
+          <t>Damson Tree</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
+          <t>Prunus domestica subsp. insititia (cultivar to confirm)</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>Light to full shade, sheltered from harsh sun and drying wind.</t>
+          <t>Full sun for reliable blossom and fruit ripening.</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>Keep the shared compost consistently moist but well drained, preferably using rainwater.</t>
+          <t>Water deeply during prolonged dry spells, especially from fruit set to harvest.</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>Mulch or top-dress with leaf mould or ericaceous compost. Prune only lightly after flowering and keep ivy stems away from its crown.</t>
+          <t>Prune only in dry summer weather to reduce silver-leaf and canker risk; remove suckers from below the graft.</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>Glossy evergreen foliage, fragrant ivory spring flowers and long-lasting red berries from autumn into winter.</t>
+          <t>White spring blossom followed by blue-black damsons in late summer or early autumn.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Skimmia Pot</t>
+          <t>Front Gate Tree</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Hedera helix 'Yellow Ripple'</t>
+          <t>Weeping Crab Apple (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Hedera helix 'Golden Starlight' (Yellow Ripple)</t>
+          <t>Malus (weeping cultivar; 'Red Jade' is a best-fit possibility)</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>Full shade to partial shade; shelter pale margins from scorching sun.</t>
+          <t>Full sun for the best blossom, fruit colour and balanced growth.</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>Share the Skimmia's evenly moist, well-drained compost; check beneath the foliage before watering.</t>
+          <t>Water deeply during prolonged drought, particularly while establishing and while fruit is swelling.</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>Trim to keep the ivy within the pot and away from the Skimmia crown. Remove any all-green reverted shoots at their origin.</t>
+          <t>Remove dead, damaged and crossing wood in winter, preserving the natural weeping framework. Record blossom and ripe-fruit details before naming the cultivar.</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>Evergreen lobed leaves with yellow-to-cream margins provide year-round trailing colour.</t>
+          <t>Spring blossom followed by small ornamental crab apples that can persist into autumn and winter.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Bed 2/3 Wall Pot</t>
+          <t>House · Hallway · Kentia Palm</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Viburnum 'Lisarose'</t>
+          <t>Kentia Palm — assumed</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Viburnum tinus 'Lisarose'</t>
+          <t>Howea forsteriana</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>Sun, partial shade or shade, sheltered from cold drying winds.</t>
+          <t>Bright indirect light; protect the fronds from strong direct sun.</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist while establishing; never leave the container waterlogged.</t>
+          <t>Check the upper few centimetres of compost before watering, then drain fully and empty the white cachepot.</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>Use humus-rich, well-drained compost. Prune only after flowering if its size needs controlling.</t>
+          <t>Maintain moderate humidity, keep away from cold draughts and radiators, and feed monthly during active spring and summer growth.</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>Brick-red winter buds open to pink-and-white flowers, followed by dark blue ornamental berries.</t>
+          <t>Evergreen indoor foliage throughout the year; growth slows as light levels fall in winter.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>Bed 2/3 Wall Pot</t>
+          <t>House · Sitting Room · ‘Gioia’ Fern</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>Vinca minor 'Illumination'</t>
+          <t>Bird’s Nest Fern ‘Gioia’</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Vinca minor 'Illumination'</t>
+          <t>Asplenium antiquum ‘Gioia’</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>Sun to shade; foliage colours best in bright indirect light or partial shade.</t>
+          <t>Bright, indirect light; protect the fronds from direct sun through the glass.</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>Moderate. Let the surface dry slightly without allowing the pot to dry completely.</t>
+          <t>Keep compost lightly moist but never saturated; water around the pot edge rather than into the centre rosette.</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>Trim trailing stems to shape and keep drainage holes clear. Do not plant into open ground without a spread plan.</t>
+          <t>Give it steady warmth and higher humidity, removing only damaged fronds at the base.</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>Golden evergreen foliage with narrow green margins and violet-blue flowers from spring into autumn.</t>
+          <t>Evergreen indoor foliage throughout the year; growth slows in lower winter light.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
+          <t>House · Hallway · Staghorn Fern</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Staghorn Fern</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Platycerium bifurcatum</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>Bright, indirect light; avoid harsh midday sun and cold draughts.</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>Check the growing medium before watering and let excess water drain completely; never keep the base wet.</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>Maintain moderate humidity and keep the fern clear of direct radiator heat. Leave the brown papery shield fronds in place.</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>Evergreen antler-like fronds are the display throughout the year; growth is slower in winter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>Skimmia Pot</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Skimmia 'Cleopatra'</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>Light to full shade, sheltered from harsh sun and drying wind.</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>Keep the shared compost consistently moist but well drained, preferably using rainwater.</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>Mulch or top-dress with leaf mould or ericaceous compost. Prune only lightly after flowering and keep ivy stems away from its crown.</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>Glossy evergreen foliage, fragrant ivory spring flowers and long-lasting red berries from autumn into winter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>Skimmia Pot</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Skimmia 'Antarctica'</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Skimmia 'Antarctica'</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>Partial to full shade, sheltered from harsh sun and drying wind.</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>Keep compost evenly moist and freely drained; rainwater is preferred where practical.</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>Use ericaceous compost and prune only lightly after flowering. Do not let the root ball dry out while establishing.</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>Glossy evergreen foliage and spring flower buds give year-round structure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>Skimmia Pot</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>Viola 'Rocky Purple Picotee' (3 plants)</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Viola cornuta 'Rocky Purple Picotee'</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>Sun to partial shade.</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>Keep the shared compost evenly moist but well drained.</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>Deadhead faded flowers and seed pods regularly to prolong flowering.</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>Purple flowers with pale picotee margins through the cool season.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>Bed 2/3 Wall Pot</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>Viburnum 'Lisarose'</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>Viburnum tinus 'Lisarose'</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>Sun, partial shade or shade, sheltered from cold drying winds.</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>Keep evenly moist while establishing; never leave the container waterlogged.</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>Use humus-rich, well-drained compost. Prune only after flowering if its size needs controlling.</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>Brick-red winter buds open to pink-and-white flowers, followed by dark blue ornamental berries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>Bed 2/3 Wall Pot</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Vinca minor 'Illumination'</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>Vinca minor 'Illumination'</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>Sun to shade; foliage colours best in bright indirect light or partial shade.</t>
+        </is>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>Moderate. Let the surface dry slightly without allowing the pot to dry completely.</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>Trim trailing stems to shape and keep drainage holes clear. Do not plant into open ground without a spread plan.</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>Golden evergreen foliage with narrow green margins and violet-blue flowers from spring into autumn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
           <t>Viburnum Pot</t>
         </is>
       </c>
-      <c r="B164" s="2" t="inlineStr">
+      <c r="B170" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus Spirit</t>
         </is>
       </c>
-      <c r="C164" s="2" t="inlineStr">
+      <c r="C170" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus 'Anvi' (Spirit)</t>
         </is>
       </c>
-      <c r="D164" s="2" t="inlineStr">
+      <c r="D170" s="2" t="inlineStr">
         <is>
           <t>Sun or partial shade, with shelter from cold drying winds.</t>
         </is>
       </c>
-      <c r="E164" s="2" t="inlineStr">
+      <c r="E170" s="2" t="inlineStr">
         <is>
           <t>Keep evenly moist but well drained while establishing; check the pot through dry and windy weather.</t>
         </is>
       </c>
-      <c r="F164" s="2" t="inlineStr">
+      <c r="F170" s="2" t="inlineStr">
         <is>
           <t>Prune only after flowering if needed. Refresh the top compost in spring and protect the container during prolonged severe cold.</t>
         </is>
       </c>
-      <c r="G164" s="2" t="inlineStr">
+      <c r="G170" s="2" t="inlineStr">
         <is>
           <t>Pink buds open to lightly fragrant creamy-white flowers from late winter into spring, followed by blue-black ornamental berries.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G164"/>
+  <autoFilter ref="A1:G170"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Present hanging baskets as paired collection
</commit_message>
<xml_diff>
--- a/Oak_Lodge_Garden_Plant_Guide.xlsx
+++ b/Oak_Lodge_Garden_Plant_Guide.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plant Guide" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$G$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$G$165</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Plant Guide'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G170"/>
+  <dimension ref="A1:G165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3861,32 +3861,32 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Trailing Fuchsia</t>
+          <t>Calluna Trio Mix (2 plants)</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Fuchsia (trailing cultivar)</t>
+          <t>Calluna vulgaris mixed cultivars</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Partial shade to full sun.</t>
+          <t>Full sun to light partial shade.</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Daily in hot weather; never let dry out completely.</t>
+          <t>Keep compost lightly moist while establishing; never waterlog.</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Feed weekly. Deadhead spent flowers. Not frost-hardy — replace each year.</t>
+          <t>Use free-draining, preferably ericaceous compost. Trim lightly after flowering, never into bare wood.</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Pendant bicolour flowers June–October.</t>
+          <t>Evergreen foliage and late-summer to autumn colour.</t>
         </is>
       </c>
     </row>
@@ -3898,12 +3898,12 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Bacopa</t>
+          <t>Viola 'Rocky Purple Picotee' (2 plants)</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Sutera cordata</t>
+          <t>Viola cornuta 'Rocky Purple Picotee'</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -3913,17 +3913,17 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist.</t>
+          <t>Keep compost evenly moist, particularly in windy weather.</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Self-cleaning; no deadheading needed. Trim back if leggy. Tender annual.</t>
+          <t>Deadhead faded flowers and seed pods to extend the display.</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Tiny white flowers May–October; neat trailing habit.</t>
+          <t>Purple flowers with a pale picotee edge through the cool season.</t>
         </is>
       </c>
     </row>
@@ -3935,32 +3935,32 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Trailing Lobelia</t>
+          <t>Hedera helix 'Yellow Ripple' (2 plants)</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Lobelia erinus (trailing)</t>
+          <t>Hedera helix 'Golden Starlight' (Yellow Ripple)</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Shade to sun; avoid prolonged scorching sun on pale foliage.</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Keep moist; hates drying out.</t>
+          <t>Keep the shared basket compost evenly moist and well drained.</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Trim back mid-season if it gets straggly. Tender annual.</t>
+          <t>Trim trails to shape and keep stems clear of neighbouring crowns.</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Blue trailing flowers May–October.</t>
+          <t>Evergreen variegated trails give structure through winter.</t>
         </is>
       </c>
     </row>
@@ -3972,32 +3972,32 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Trailing Verbena</t>
+          <t>Pansy 'Fire' (2 plants)</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Verbena (trailing cultivar)</t>
+          <t>Viola × wittrockiana 'Fire'</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Regular; don't let dry out.</t>
+          <t>Keep evenly moist but never saturated.</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Deadhead to extend flowering. Tender annual.</t>
+          <t>Remove faded flowers and seed pods regularly.</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Clusters of flowers June–October.</t>
+          <t>Cool-season flowers provide autumn-to-spring colour.</t>
         </is>
       </c>
     </row>
@@ -4009,661 +4009,661 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Petunia</t>
+          <t>Pansy 'Rose Surprise' (2 plants)</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Petunia (cultivar unknown)</t>
+          <t>Viola × wittrockiana 'Rose Surprise'</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Check daily in warm weather; water thoroughly before the basket dries out.</t>
+          <t>Keep evenly moist but never saturated.</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Feed weekly during flowering and remove faded blooms and seed capsules. Trim bare stems back to leafy growth.</t>
+          <t>Remove faded flowers and seed pods regularly.</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Funnel-shaped summer flowers from June until the first frost; cultivar unresolved.</t>
+          <t>Cool-season flowers provide autumn-to-spring colour.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Baskets</t>
+          <t>Front Bed 1</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Calluna Trio Mix (2 plants)</t>
+          <t>Hydrangea</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Calluna vulgaris mixed cultivars</t>
+          <t>Hydrangea macrophylla</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade.</t>
+          <t>Morning sun, afternoon shade.</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Keep compost lightly moist while establishing; never waterlog.</t>
+          <t>Thirsty — water well in dry spells.</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Use free-draining, preferably ericaceous compost. Trim lightly after flowering, never into bare wood.</t>
+          <t>Leave old flower heads over winter; prune to a strong bud in spring.</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Evergreen foliage and late-summer to autumn colour.</t>
+          <t>Mophead flowers July–Sept; bare in winter.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Baskets</t>
+          <t>Front Bed 1</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Viola 'Rocky Purple Picotee' (2 plants)</t>
+          <t>Lavender</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Viola cornuta 'Rocky Purple Picotee'</t>
+          <t>Lavandula angustifolia</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Full sun.</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Keep compost evenly moist, particularly in windy weather.</t>
+          <t>Drought-tolerant.</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Deadhead faded flowers and seed pods to extend the display.</t>
+          <t>Trim after flowering and again in spring; don't cut into old wood.</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Purple flowers with a pale picotee edge through the cool season.</t>
+          <t>Purple spikes June–Aug; aromatic year-round.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Baskets</t>
+          <t>Front Bed 2</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Hedera helix 'Yellow Ripple' (2 plants)</t>
+          <t>Coprosma 'Inferno'</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Hedera helix 'Golden Starlight' (Yellow Ripple)</t>
+          <t>Coprosma 'Inferno'</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Shade to sun; avoid prolonged scorching sun on pale foliage.</t>
+          <t>Full sun to partial shade; stronger light brings out the warm foliage colour.</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Keep the shared basket compost evenly moist and well drained.</t>
+          <t>Moderate while establishing. Avoid waterlogged soil.</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Trim trails to shape and keep stems clear of neighbouring crowns.</t>
+          <t>Shelter from cold drying winds and protect in severe frost. Trim lightly in spring to keep a compact shape.</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Evergreen variegated trails give structure through winter.</t>
+          <t>Glossy green, cream, orange and red foliage intensifies in cooler weather; evergreen in a sheltered spot.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Baskets</t>
+          <t>Front Bed 2</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Pansy 'Fire' (2 plants)</t>
+          <t>Coprosma 'Pina Colada'</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Viola × wittrockiana 'Fire'</t>
+          <t>Coprosma 'Pina Colada'</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Full sun to partial shade; best colour in a bright, sheltered position.</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist but never saturated.</t>
+          <t>Moderate while establishing. Let the soil drain between waterings.</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Remove faded flowers and seed pods regularly.</t>
+          <t>Protect from severe frost and cold winds. Lightly trim any untidy growth in spring.</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Cool-season flowers provide autumn-to-spring colour.</t>
+          <t>Golden foliage develops orange and bronze tones through autumn and winter; evergreen when sheltered.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Baskets</t>
+          <t>Front Bed 2</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Pansy 'Rose Surprise' (2 plants)</t>
+          <t>Coprosma 'City Knights'</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Viola × wittrockiana 'Rose Surprise'</t>
+          <t>Coprosma 'City Knights'</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Full sun to partial shade; bright shelter gives the richest leaf colour.</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist but never saturated.</t>
+          <t>Moderate while establishing. Keep the root zone drained and do not allow prolonged drought in its first season.</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Remove faded flowers and seed pods regularly.</t>
+          <t>Protect from severe frost and cold drying winds. Remove only damaged tips in spring and avoid forcing soft late growth with autumn feed.</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Cool-season flowers provide autumn-to-spring colour.</t>
+          <t>Glossy evergreen foliage holds deep burgundy, red and dark green tones, strengthening the bed's winter colour.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 1</t>
+          <t>Front Bed 2</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Hydrangea</t>
+          <t>Hebe 'Kiwi' (Horopito)</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Hydrangea macrophylla</t>
+          <t>Hebe 'Kiwi'</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Morning sun, afternoon shade.</t>
+          <t>Full sun to partial shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Thirsty — water well in dry spells.</t>
+          <t>Moderate while establishing; avoid waterlogged winter soil.</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Leave old flower heads over winter; prune to a strong bud in spring.</t>
+          <t>Deadhead faded spikes and trim lightly after flowering. Avoid cutting back into old bare wood.</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Mophead flowers July–Sept; bare in winter.</t>
+          <t>Purple flower spikes in summer above glossy green leaves with dark new growth; evergreen.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 1</t>
+          <t>Front Bed 2</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Lavender</t>
+          <t>Polemonium 'Golden Feathers'</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Lavandula angustifolia</t>
+          <t>Polemonium 'Golden Feathers'</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Sun to partial shade; give afternoon shade in hot weather.</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Drought-tolerant.</t>
+          <t>Moderate. Keep evenly moist but not waterlogged while establishing.</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Trim after flowering and again in spring; don't cut into old wood.</t>
+          <t>Deadhead after flowering and cut tired foliage back for fresh growth. Watch for powdery mildew in dry, crowded conditions.</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Purple spikes June–Aug; aromatic year-round.</t>
+          <t>Gold-edged ferny foliage from spring; lilac-mauve bell flowers in spring and early summer; herbaceous in winter.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 2</t>
+          <t>Front Bed 3</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'Inferno'</t>
+          <t>Climbing Rose 'Super Fairy'</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'Inferno'</t>
+          <t>Rosa 'Helsufair'</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; stronger light brings out the warm foliage colour.</t>
+          <t>Sun to light partial shade.</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Moderate while establishing. Avoid waterlogged soil.</t>
+          <t>Deep water at the base in dry spells, especially while establishing.</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>Shelter from cold drying winds and protect in severe frost. Trim lightly in spring to keep a compact shape.</t>
+          <t>Vigorous climber to about 2.5m high and 1.5m wide. Tie long shoots into the wall support and fan laterals out. Prune in late winter and deadhead after flowering.</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>Glossy green, cream, orange and red foliage intensifies in cooler weather; evergreen in a sheltered spot.</t>
+          <t>Clusters of small, light-pink double flowers from June into autumn; deciduous in winter.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 2</t>
+          <t>Front Bed 3</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'Pina Colada'</t>
+          <t>Variegated Dogwood</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'Pina Colada'</t>
+          <t>Cornus alba 'Elegantissima'</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; best colour in a bright, sheltered position.</t>
+          <t>Sun or partial shade; the leaf colour and winter stems are strongest in good light.</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Moderate while establishing. Let the soil drain between waterings.</t>
+          <t>Moisture-loving. Water deeply while it re-establishes and during prolonged dry spells.</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>Protect from severe frost and cold winds. Lightly trim any untidy growth in spring.</t>
+          <t>Mulch after planting. Once settled, remove about a third of the oldest stems at the base in March to encourage vivid new winter stems.</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Golden foliage develops orange and bronze tones through autumn and winter; evergreen when sheltered.</t>
+          <t>Cream-edged leaves spring–autumn; brilliant red stems provide the main display in winter.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 2</t>
+          <t>Front Bed 3</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'City Knights'</t>
+          <t>Red Hot Poker</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Coprosma 'City Knights'</t>
+          <t>Kniphofia</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; bright shelter gives the richest leaf colour.</t>
+          <t>Full sun for the strongest flowering.</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Moderate while establishing. Keep the root zone drained and do not allow prolonged drought in its first season.</t>
+          <t>Moderate while re-establishing; drought-tolerant once rooted, but dislikes winter waterlogging.</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Protect from severe frost and cold drying winds. Remove only damaged tips in spring and avoid forcing soft late growth with autumn feed.</t>
+          <t>Keep the crown clear and well drained. Remove spent flower stems, tidy old foliage in spring and divide congested clumps every four or five years.</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>Glossy evergreen foliage holds deep burgundy, red and dark green tones, strengthening the bed's winter colour.</t>
+          <t>Bold orange-red poker spikes July–September above strappy, mostly evergreen foliage.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 2</t>
+          <t>Front Bed 3</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Hebe 'Kiwi' (Horopito)</t>
+          <t>Leucothoe 'Little Flames'</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Hebe 'Kiwi'</t>
+          <t>Leucothoe 'Little Flames'</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a sheltered position.</t>
+          <t>Full sun to partial shade; some shade helps the soil stay evenly moist.</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Moderate while establishing; avoid waterlogged winter soil.</t>
+          <t>Keep moist but well drained, especially while establishing. Use rainwater where practical.</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>Deadhead faded spikes and trim lightly after flowering. Avoid cutting back into old bare wood.</t>
+          <t>Needs acidic soil. Mulch with leaf mould or composted bark and prune only to remove damaged growth or lightly reshape after flowering.</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>Purple flower spikes in summer above glossy green leaves with dark new growth; evergreen.</t>
+          <t>Evergreen leaves and stems flush vivid red when young, with clusters of small white urn-shaped flowers in spring.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 2</t>
+          <t>Front Bed 3</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Polemonium 'Golden Feathers'</t>
+          <t>Rose (pink)</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Polemonium 'Golden Feathers'</t>
+          <t>Rosa — IDENTIFY</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade; give afternoon shade in hot weather.</t>
+          <t>Sun.</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Moderate. Keep evenly moist but not waterlogged while establishing.</t>
+          <t>Deep watering, mulch in spring.</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>Deadhead after flowering and cut tired foliage back for fresh growth. Watch for powdery mildew in dry, crowded conditions.</t>
+          <t>Prune late winter; deadhead through summer.</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Gold-edged ferny foliage from spring; lilac-mauve bell flowers in spring and early summer; herbaceous in winter.</t>
+          <t>Flowers June–Sept; bare winter.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 3</t>
+          <t>Front Bed 4</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Climbing Rose 'Super Fairy'</t>
+          <t>Photinia (existing canopy)</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Rosa 'Helsufair'</t>
+          <t>Photinia (cultivar to confirm)</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Sun to light partial shade.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Deep water at the base in dry spells, especially while establishing.</t>
+          <t>Water deeply only in prolonged dry periods once established.</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>Vigorous climber to about 2.5m high and 1.5m wide. Tie long shoots into the wall support and fan laterals out. Prune in late winter and deadhead after flowering.</t>
+          <t>Lightly prune after the spring flush if shaping is needed. Keep the new underplanting mulched and watered while it establishes around the existing roots.</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>Clusters of small, light-pink double flowers from June into autumn; deciduous in winter.</t>
+          <t>Evergreen canopy; fresh growth is often bronze-red and white flower clusters can appear in spring.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 3</t>
+          <t>Front Bed 4</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>Variegated Dogwood</t>
+          <t>The Pilgrim</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Cornus alba 'Elegantissima'</t>
+          <t>Rosa 'Auswalker'</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Sun or partial shade; the leaf colour and winter stems are strongest in good light.</t>
+          <t>Full sun to light partial shade. Aim for at least four hours of direct sun.</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>Moisture-loving. Water deeply while it re-establishes and during prolonged dry spells.</t>
+          <t>Deep water at the base during dry spells, especially while establishing.</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>Mulch after planting. Once settled, remove about a third of the oldest stems at the base in March to encourage vivid new winter stems.</t>
+          <t>David Austin medium climber. Tie new canes into the support, fanning them horizontally where possible. Feed and mulch in spring; deadhead through summer; prune in late winter.</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>Cream-edged leaves spring–autumn; brilliant red stems provide the main display in winter.</t>
+          <t>Soft yellow, rosette-shaped flowers with a tea fragrance from June into autumn; deciduous in winter.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 3</t>
+          <t>Front Bed 4</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Red Hot Poker</t>
+          <t>The Generous Gardener</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Kniphofia</t>
+          <t>Rosa 'Ausdrawn'</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Full sun for the strongest flowering.</t>
+          <t>Full sun to light partial shade. Tolerates a little less sun than many climbing roses.</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>Moderate while re-establishing; drought-tolerant once rooted, but dislikes winter waterlogging.</t>
+          <t>Deep water at the base during dry spells, especially in its first two years.</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>Keep the crown clear and well drained. Remove spent flower stems, tidy old foliage in spring and divide congested clumps every four or five years.</t>
+          <t>David Austin medium climber. Train and tie in long shoots, feed and mulch in spring, deadhead repeat flowers and prune in late winter. Good disease resistance.</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>Bold orange-red poker spikes July–September above strappy, mostly evergreen foliage.</t>
+          <t>Pale pink, cup-shaped flowers fading almost white, with a strong old-rose and musk fragrance; repeat flowers June–autumn.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 3</t>
+          <t>Front Bed 4</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>Leucothoe 'Little Flames'</t>
+          <t>Physocarpus Cluster 1 (2 × Little Devil + 1 × Lady in Red)</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>Leucothoe 'Little Flames'</t>
+          <t>Physocarpus opulifolius 'Little Devil' &amp; 'Lady in Red'</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; some shade helps the soil stay evenly moist.</t>
+          <t>Sun to partial shade; foliage is darkest with good light.</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>Keep moist but well drained, especially while establishing. Use rainwater where practical.</t>
+          <t>Sprinkler supplied. Check all three root balls through establishment and water deeply in dry spells.</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>Needs acidic soil. Mulch with leaf mould or composted bark and prune only to remove damaged growth or lightly reshape after flowering.</t>
+          <t>Keep all three crowns distinct, with the taller Lady in Red rising through the two compact Little Devils. Renew individual shrubs from the base only when mature and congested.</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>Evergreen leaves and stems flush vivid red when young, with clusters of small white urn-shaped flowers in spring.</t>
+          <t>Burgundy and red-bronze foliage spring to autumn with pale pink flower clusters in early summer; bare in winter.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 3</t>
+          <t>Front Bed 4</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Rose (pink)</t>
+          <t>Physocarpus Cluster 2 (2 × Lady in Red + 1 × Little Devil)</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Rosa — IDENTIFY</t>
+          <t>Physocarpus opulifolius 'Lady in Red' &amp; 'Little Devil'</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Sun.</t>
+          <t>Sun to partial shade; best foliage colour in brighter light.</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>Deep watering, mulch in spring.</t>
+          <t>Sprinkler supplied. Check all three root balls through establishment and water deeply in dry spells.</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>Prune late winter; deadhead through summer.</t>
+          <t>Keep the compact Little Devil readable against the two taller Lady in Reds. Remove a few oldest stems at the base only when congestion develops.</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>Flowers June–Sept; bare winter.</t>
+          <t>Red, bronze and burgundy foliage spring to autumn with pink flower clusters in summer; bare in winter.</t>
         </is>
       </c>
     </row>
@@ -4675,32 +4675,32 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>Photinia (existing canopy)</t>
+          <t>Azalea japonica 'Silvester'</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>Photinia (cultivar to confirm)</t>
+          <t>Rhododendron 'Sylvester'</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Partial or dappled shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>Water deeply only in prolonged dry periods once established.</t>
+          <t>Dropper supplied. Keep its shallow acidic root zone evenly moist, preferably with rainwater.</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>Lightly prune after the spring flush if shaping is needed. Keep the new underplanting mulched and watered while it establishes around the existing roots.</t>
+          <t>Grow shallowly in acidic, humus-rich soil and mulch with leaf mould. Deadhead carefully after flowering and prune only damaged or wayward growth.</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>Evergreen canopy; fresh growth is often bronze-red and white flower clusters can appear in spring.</t>
+          <t>Compact evergreen foliage with purple-pink flowers in late spring.</t>
         </is>
       </c>
     </row>
@@ -4712,32 +4712,32 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>The Pilgrim</t>
+          <t>Nemesia 'Lady Penelope'</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Rosa 'Auswalker'</t>
+          <t>Nemesia 'Lady Penelope' (best-fit identification)</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade. Aim for at least four hours of direct sun.</t>
+          <t>Full sun to light partial shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>Deep water at the base during dry spells, especially while establishing.</t>
+          <t>Dropper supplied. Keep evenly moist while flowering but never waterlogged.</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>David Austin medium climber. Tie new canes into the support, fanning them horizontally where possible. Feed and mulch in spring; deadhead through summer; prune in late winter.</t>
+          <t>Trim tired flowering stems by about a third for another flush. Feed lightly while flowering and protect from frost.</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>Soft yellow, rosette-shaped flowers with a tea fragrance from June into autumn; deciduous in winter.</t>
+          <t>Fragrant rose-pink and white flowers with pink markings and a yellow eye from late spring into autumn.</t>
         </is>
       </c>
     </row>
@@ -4749,32 +4749,32 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>The Generous Gardener</t>
+          <t>Purple Gem</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>Rosa 'Ausdrawn'</t>
+          <t>Sarcococca hookeriana var. humilis 'Purple Gem'</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade. Tolerates a little less sun than many climbing roses.</t>
+          <t>Shade to partial shade.</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>Deep water at the base during dry spells, especially in its first two years.</t>
+          <t>Water in dry spells while establishing; tolerates dry shade once settled.</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>David Austin medium climber. Train and tie in long shoots, feed and mulch in spring, deadhead repeat flowers and prune in late winter. Good disease resistance.</t>
+          <t>Evergreen winter-scented shrub. Keep ivy from engulfing it and prune only lightly after flowering if needed.</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>Pale pink, cup-shaped flowers fading almost white, with a strong old-rose and musk fragrance; repeat flowers June–autumn.</t>
+          <t>Glossy evergreen foliage and purple young stems; small fragrant winter flowers followed by dark berries.</t>
         </is>
       </c>
     </row>
@@ -4786,32 +4786,32 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Physocarpus Cluster 1 (2 × Little Devil + 1 × Lady in Red)</t>
+          <t>Rhododendron 'Libretto'</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>Physocarpus opulifolius 'Little Devil' &amp; 'Lady in Red'</t>
+          <t>Rhododendron 'Libretto'</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade; foliage is darkest with good light.</t>
+          <t>Light dappled shade, sheltered from cold drying wind and harsh early-morning sun.</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>Sprinkler supplied. Check all three root balls through establishment and water deeply in dry spells.</t>
+          <t>Keep the shallow root zone evenly moist but never waterlogged. Prefer rainwater, especially in hard-water areas.</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>Keep all three crowns distinct, with the taller Lady in Red rising through the two compact Little Devils. Renew individual shrubs from the base only when mature and congested.</t>
+          <t>Plant shallowly in acidic, humus-rich soil. Mulch with composted bark while keeping the stem clear; deadhead carefully and prune only dead or wayward growth after flowering.</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>Burgundy and red-bronze foliage spring to autumn with pale pink flower clusters in early summer; bare in winter.</t>
+          <t>Evergreen foliage all year; large dark-purple flowers with an olive-yellow flare in late May and early June.</t>
         </is>
       </c>
     </row>
@@ -4823,32 +4823,32 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>Physocarpus Cluster 2 (2 × Lady in Red + 1 × Little Devil)</t>
+          <t>Festuca 'Elijah Blue' (3 plants)</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>Physocarpus opulifolius 'Lady in Red' &amp; 'Little Devil'</t>
+          <t>Festuca glauca 'Elijah Blue'</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade; best foliage colour in brighter light.</t>
+          <t>Full sun to light partial shade.</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>Sprinkler supplied. Check all three root balls through establishment and water deeply in dry spells.</t>
+          <t>Water regularly during the first season; drought tolerant once established.</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>Keep the compact Little Devil readable against the two taller Lady in Reds. Remove a few oldest stems at the base only when congestion develops.</t>
+          <t>Comb out dead leaves in spring and divide congested clumps every few years. Do not routinely shear hard.</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>Red, bronze and burgundy foliage spring to autumn with pink flower clusters in summer; bare in winter.</t>
+          <t>Blue-grey, mostly evergreen foliage for year-round texture; airy flower stems in early summer.</t>
         </is>
       </c>
     </row>
@@ -4860,32 +4860,32 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Azalea japonica 'Silvester'</t>
+          <t>Pieris 'Polar Passion'</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>Rhododendron 'Sylvester'</t>
+          <t>Pieris japonica 'Ppobas' (Polar Passion)</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Partial or dappled shade in a sheltered position.</t>
+          <t>Partial shade, sheltered from cold winds and harsh early sun.</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>Dropper supplied. Keep its shallow acidic root zone evenly moist, preferably with rainwater.</t>
+          <t>Keep evenly moist in acidic, well-drained soil; use rainwater where practical.</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>Grow shallowly in acidic, humus-rich soil and mulch with leaf mould. Deadhead carefully after flowering and prune only damaged or wayward growth.</t>
+          <t>Mulch with ericaceous material and remove only spent flowers or damaged stems. Do not apply lime.</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>Compact evergreen foliage with purple-pink flowers in late spring.</t>
+          <t>Colourful young foliage and hanging clusters of spring flowers above evergreen leaves.</t>
         </is>
       </c>
     </row>
@@ -4897,32 +4897,32 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>Nemesia 'Lady Penelope'</t>
+          <t>Dahlia 'Tampico'</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Nemesia 'Lady Penelope' (best-fit identification)</t>
+          <t>Dahlia Dalina Maxi Tampico ('Datretten')</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade in a sheltered position.</t>
+          <t>Full sun, sheltered from strong wind.</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>Dropper supplied. Keep evenly moist while flowering but never waterlogged.</t>
+          <t>Water deeply whenever the upper soil begins to dry; do not leave the tuber in saturated ground.</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>Trim tired flowering stems by about a third for another flush. Feed lightly while flowering and protect from frost.</t>
+          <t>Deadhead to keep flowers coming and support stems if they begin to lean. Lift and store the tuber frost-free after the first frost, or protect it with a deep dry mulch in a mild winter.</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>Fragrant rose-pink and white flowers with pink markings and a yellow eye from late spring into autumn.</t>
+          <t>Red-and-white decorative flowers from summer until frost; dormant tuber in winter.</t>
         </is>
       </c>
     </row>
@@ -4934,32 +4934,32 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Purple Gem</t>
+          <t>Verbena 'Margaret's Memory'</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>Sarcococca hookeriana var. humilis 'Purple Gem'</t>
+          <t>Glandularia 'Margaret's Memory'</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Shade to partial shade.</t>
+          <t>Full sun to light partial shade.</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>Water in dry spells while establishing; tolerates dry shade once settled.</t>
+          <t>Keep moist but well drained while establishing; avoid waterlogged winter soil.</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>Evergreen winter-scented shrub. Keep ivy from engulfing it and prune only lightly after flowering if needed.</t>
+          <t>Deadhead or cut back after a flower flush. Take late-summer tip cuttings as insurance where winter cold or wet is severe.</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>Glossy evergreen foliage and purple young stems; small fragrant winter flowers followed by dark berries.</t>
+          <t>Lilac-pink flowers with dark eyes from spring into late autumn; semi-evergreen in a sheltered winter.</t>
         </is>
       </c>
     </row>
@@ -4971,32 +4971,32 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>Rhododendron 'Libretto'</t>
+          <t>Calluna Trio Mix (2 plants)</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>Rhododendron 'Libretto'</t>
+          <t>Calluna vulgaris mixed cultivars</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Light dappled shade, sheltered from cold drying wind and harsh early-morning sun.</t>
+          <t>Full sun in an open position.</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>Keep the shallow root zone evenly moist but never waterlogged. Prefer rainwater, especially in hard-water areas.</t>
+          <t>Sprinkler supplied; keep the root zone moist while establishing but never waterlogged.</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>Plant shallowly in acidic, humus-rich soil. Mulch with composted bark while keeping the stem clear; deadhead carefully and prune only dead or wayward growth after flowering.</t>
+          <t>Keep the soil acidic and free draining. Trim lightly after flowering, never back into bare old wood, and keep fallen leaves clear of the crowns.</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>Evergreen foliage all year; large dark-purple flowers with an olive-yellow flare in late May and early June.</t>
+          <t>A two-plant mixed Calluna group with pink, white and lime-green flower-and-foliage interest from late summer into autumn.</t>
         </is>
       </c>
     </row>
@@ -5008,32 +5008,32 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Festuca 'Elijah Blue' (3 plants)</t>
+          <t>Achillea</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>Festuca glauca 'Elijah Blue'</t>
+          <t>Achillea millefolium</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade.</t>
+          <t>Full sun.</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>Water regularly during the first season; drought tolerant once established.</t>
+          <t>Low to moderate. Drought-tolerant once established.</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>Comb out dead leaves in spring and divide congested clumps every few years. Do not routinely shear hard.</t>
+          <t>Cut back after first flush for a second showing. Divide clumps every 2–3 years to keep vigorous. Good for cutting.</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>Blue-grey, mostly evergreen foliage for year-round texture; airy flower stems in early summer.</t>
+          <t>Flat-headed flower clusters in red, pink or yellow June–September; feathery aromatic foliage through the season.</t>
         </is>
       </c>
     </row>
@@ -5045,217 +5045,217 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>Pieris 'Polar Passion'</t>
+          <t>Azalea japonica 'Lotte'</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>Pieris japonica 'Ppobas' (Polar Passion)</t>
+          <t>Rhododendron 'Lotte'</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>Partial shade, sheltered from cold winds and harsh early sun.</t>
+          <t>Partial or dappled shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist in acidic, well-drained soil; use rainwater where practical.</t>
+          <t>Dropper supplied. Keep its shallow acidic root zone evenly moist, preferably with rainwater.</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>Mulch with ericaceous material and remove only spent flowers or damaged stems. Do not apply lime.</t>
+          <t>Grow shallowly in acidic, humus-rich soil and mulch with leaf mould. Deadhead carefully after flowering and prune only damaged growth.</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>Colourful young foliage and hanging clusters of spring flowers above evergreen leaves.</t>
+          <t>Compact glossy evergreen foliage with deep-pink flowers in late spring.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 4</t>
+          <t>Front Bed 5</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Dahlia 'Tampico'</t>
+          <t>Mexican Orange Blossom</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>Dahlia Dalina Maxi Tampico ('Datretten')</t>
+          <t>Choisya ternata 'Sundance'</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Full sun, sheltered from strong wind.</t>
+          <t>Sun for best colour.</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>Water deeply whenever the upper soil begins to dry; do not leave the tuber in saturated ground.</t>
+          <t>Moderate.</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>Deadhead to keep flowers coming and support stems if they begin to lean. Lift and store the tuber frost-free after the first frost, or protect it with a deep dry mulch in a mild winter.</t>
+          <t>Light prune after flowering to shape. Low-care.</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>Red-and-white decorative flowers from summer until frost; dormant tuber in winter.</t>
+          <t>Golden evergreen foliage; scented white flowers spring &amp; again autumn.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 4</t>
+          <t>Front Bed 5</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>Verbena 'Margaret's Memory'</t>
+          <t>Shrub Rose (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>Glandularia 'Margaret's Memory'</t>
+          <t>Rosa (Shrub Group; cultivar to confirm)</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade.</t>
+          <t>Full sun for the strongest flowering; tolerates light partial shade.</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>Keep moist but well drained while establishing; avoid waterlogged winter soil.</t>
+          <t>Water deeply in sustained dry spells, especially while flowering and forming hips.</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>Deadhead or cut back after a flower flush. Take late-summer tip cuttings as insurance where winter cold or wet is severe.</t>
+          <t>Remove dead, damaged and crossing stems in late winter. Thin congested growth and preserve sound hips where autumn colour and wildlife value are wanted.</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>Lilac-pink flowers with dark eyes from spring into late autumn; semi-evergreen in a sheltered winter.</t>
+          <t>Flowers are followed by red-orange rose hips — the fruits seen in the July photographs.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 4</t>
+          <t>Front Bed 5</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Calluna Trio Mix (2 plants)</t>
+          <t>Bay Tree</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>Calluna vulgaris mixed cultivars</t>
+          <t>Laurus nobilis</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Full sun in an open position.</t>
+          <t>Full sun to partial shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>Sprinkler supplied; keep the root zone moist while establishing but never waterlogged.</t>
+          <t>Water while establishing and during prolonged drought; avoid waterlogged winter soil.</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>Keep the soil acidic and free draining. Trim lightly after flowering, never back into bare old wood, and keep fallen leaves clear of the crowns.</t>
+          <t>Trim lightly in late spring or summer to retain the standard shape. Remove suckers and frost-damaged tips with secateurs.</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>A two-plant mixed Calluna group with pink, white and lime-green flower-and-foliage interest from late summer into autumn.</t>
+          <t>Aromatic evergreen leaves throughout the year; small spring flowers may be followed by dark berries on female plants.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 4</t>
+          <t>Front Bed 5</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>Achillea</t>
+          <t>Japanese Skimmia</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>Achillea millefolium</t>
+          <t>Skimmia japonica (cultivar and sex to confirm)</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Partial shade to shade; shelter from the hottest afternoon sun.</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>Low to moderate. Drought-tolerant once established.</t>
+          <t>Keep evenly moist but well drained, especially in dry summer weather.</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>Cut back after first flush for a second showing. Divide clumps every 2–3 years to keep vigorous. Good for cutting.</t>
+          <t>Mulch with leaf mould or ericaceous compost and prune only to remove damaged or awkward stems. Confirm sex and cultivar from flowers and fruit.</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>Flat-headed flower clusters in red, pink or yellow June–September; feathery aromatic foliage through the season.</t>
+          <t>Evergreen foliage and spring flower clusters; female or hermaphrodite forms can carry red berries when pollinated.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 4</t>
+          <t>Front Bed 5</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Azalea japonica 'Lotte'</t>
+          <t>Hardy Fuchsia (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>Rhododendron 'Lotte'</t>
+          <t>Fuchsia magellanica hybrid (cultivar to confirm)</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Partial or dappled shade in a sheltered position.</t>
+          <t>Full sun to partial shade, sheltered from cold drying winds.</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>Dropper supplied. Keep its shallow acidic root zone evenly moist, preferably with rainwater.</t>
+          <t>Moist but well-drained soil; water in sustained dry spells while in flower.</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>Grow shallowly in acidic, humus-rich soil and mulch with leaf mould. Deadhead carefully after flowering and prune only damaged growth.</t>
+          <t>Leave the top growth through winter, mulch the crown, then cut frost-damaged stems back to live buds in spring.</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>Compact glossy evergreen foliage with deep-pink flowers in late spring.</t>
+          <t>Pendant flowers from summer into autumn; top growth may die back in hard winters and regrow from the base.</t>
         </is>
       </c>
     </row>
@@ -5267,32 +5267,32 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>Mexican Orange Blossom</t>
+          <t>Clematis (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>Choisya ternata 'Sundance'</t>
+          <t>Clematis viticella (cultivar to confirm)</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Sun for best colour.</t>
+          <t>Sun to partial shade, with a cool shaded root run.</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>Moderate.</t>
+          <t>Keep moist but well drained; soak the root zone during prolonged drought.</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>Light prune after flowering to shape. Low-care.</t>
+          <t>Treat as pruning group 3 while the viticella identity remains the best fit: cut to strong buds 30–45cm above ground in late winter and tie in new shoots.</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>Golden evergreen foliage; scented white flowers spring &amp; again autumn.</t>
+          <t>Deciduous climber with abundant summer flowers on new growth.</t>
         </is>
       </c>
     </row>
@@ -5304,32 +5304,32 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Shrub Rose (cultivar to confirm)</t>
+          <t>Hydrangea 'Bloody Marie'</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>Rosa (Shrub Group; cultivar to confirm)</t>
+          <t>Hydrangea paniculata 'Bloody Marie'</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>Full sun for the strongest flowering; tolerates light partial shade.</t>
+          <t>Full sun to partial shade; afternoon shelter helps preserve moisture.</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>Water deeply in sustained dry spells, especially while flowering and forming hips.</t>
+          <t>Keep the root zone consistently moist while establishing and through hot dry spells.</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>Remove dead, damaged and crossing stems in late winter. Thin congested growth and preserve sound hips where autumn colour and wildlife value are wanted.</t>
+          <t>Mulch in spring and prune in late winter or early spring before new growth, retaining a sound low framework. Panicle hydrangeas flower on the current season's shoots.</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>Flowers are followed by red-orange rose hips — the fruits seen in the July photographs.</t>
+          <t>Large cream panicles age through pink toward red from July to September; deciduous in winter.</t>
         </is>
       </c>
     </row>
@@ -5341,32 +5341,32 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>Bay Tree</t>
+          <t>Euphorbia 'Ascot Petite'</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>Laurus nobilis</t>
+          <t>Euphorbia × martinii 'Ascot Petite'</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a sheltered position.</t>
+          <t>Full sun in a sheltered position.</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing and during prolonged drought; avoid waterlogged winter soil.</t>
+          <t>Water while establishing, then sparingly; sharp drainage is important in winter.</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>Trim lightly in late spring or summer to retain the standard shape. Remove suckers and frost-damaged tips with secateurs.</t>
+          <t>Remove old flowering stems at the base with gloves once replacement shoots are clear. Avoid disturbing the crown in cold wet weather.</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>Aromatic evergreen leaves throughout the year; small spring flowers may be followed by dark berries on female plants.</t>
+          <t>Compact evergreen mound with yellow-green spring and early-summer flowerheads.</t>
         </is>
       </c>
     </row>
@@ -5378,32 +5378,32 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Japanese Skimmia</t>
+          <t>Flaming Silver</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>Skimmia japonica (cultivar and sex to confirm)</t>
+          <t>Pieris japonica 'Flaming Silver'</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Partial shade to shade; shelter from the hottest afternoon sun.</t>
+          <t>Partial shade to sun, sheltered from harsh morning frost.</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist but well drained, especially in dry summer weather.</t>
+          <t>Keep evenly moist, especially in dry spells; do not let the rootball dry out.</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>Mulch with leaf mould or ericaceous compost and prune only to remove damaged or awkward stems. Confirm sex and cultivar from flowers and fruit.</t>
+          <t>Ericaceous shrub. Use rainwater where practical and mulch with ericaceous material; prune only lightly after flowering.</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>Evergreen foliage and spring flower clusters; female or hermaphrodite forms can carry red berries when pollinated.</t>
+          <t>Evergreen, cream-edged leaves with red spring growth and cream flowers in spring.</t>
         </is>
       </c>
     </row>
@@ -5415,32 +5415,32 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>Hardy Fuchsia (cultivar to confirm)</t>
+          <t>Astrantia trio</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>Fuchsia magellanica hybrid (cultivar to confirm)</t>
+          <t>Astrantia major 'Buckland', 'Claret' &amp; 'Star of Love'</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade, sheltered from cold drying winds.</t>
+          <t>Sun to light shade.</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>Moist but well-drained soil; water in sustained dry spells while in flower.</t>
+          <t>Keep consistently moist during dry weather, particularly while re-establishing.</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>Leave the top growth through winter, mulch the crown, then cut frost-damaged stems back to live buds in spring.</t>
+          <t>Mulch annually with organic matter. Deadhead to prolong flowering and cut back tired stems after flowering.</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>Pendant flowers from summer into autumn; top growth may die back in hard winters and regrow from the base.</t>
+          <t>Pin-cushion flowers in blush, soft pink and claret shades through summer; foliage dies back in winter.</t>
         </is>
       </c>
     </row>
@@ -5452,32 +5452,32 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Clematis (cultivar to confirm)</t>
+          <t>Pittosporum 'Tom Thumb'</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>Clematis viticella (cultivar to confirm)</t>
+          <t>Pittosporum tenuifolium 'Tom Thumb'</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade, with a cool shaded root run.</t>
+          <t>Full sun to partial shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>Keep moist but well drained; soak the root zone during prolonged drought.</t>
+          <t>Water while establishing; later only during prolonged drought. Avoid winter waterlogging.</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>Treat as pruning group 3 while the viticella identity remains the best fit: cut to strong buds 30–45cm above ground in late winter and tie in new shoots.</t>
+          <t>Usually needs little pruning. Remove frost-damaged tips in late spring and protect from cold drying wind.</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>Deciduous climber with abundant summer flowers on new growth.</t>
+          <t>Lime-green young leaves mature to deep purple, forming a dense rounded evergreen mound.</t>
         </is>
       </c>
     </row>
@@ -5489,32 +5489,32 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>Hydrangea 'Bloody Marie'</t>
+          <t>Gaura 'Gaudi Red'</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>Hydrangea paniculata 'Bloody Marie'</t>
+          <t>Oenothera lindheimeri 'Florgaured' (Gaudi Red)</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; afternoon shelter helps preserve moisture.</t>
+          <t>Full sun in a warm, sheltered position.</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>Keep the root zone consistently moist while establishing and through hot dry spells.</t>
+          <t>Water while establishing, then sparingly; sharp winter drainage is essential.</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>Mulch in spring and prune in late winter or early spring before new growth, retaining a sound low framework. Panicle hydrangeas flower on the current season's shoots.</t>
+          <t>Deadhead for a longer display. Leave stems over winter and cut back after the worst frosts in spring.</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>Large cream panicles age through pink toward red from July to September; deciduous in winter.</t>
+          <t>Deep pink-red flowers dance above burgundy-green foliage from summer into autumn.</t>
         </is>
       </c>
     </row>
@@ -5526,32 +5526,32 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Euphorbia 'Ascot Petite'</t>
+          <t>Heather 'Bell's Extra Special'</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>Euphorbia × martinii 'Ascot Petite'</t>
+          <t>Erica carnea 'Bell's Extra Special'</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Full sun in a sheltered position.</t>
+          <t>Full sun to light partial shade; stronger light keeps the foliage richly coloured.</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing, then sparingly; sharp drainage is important in winter.</t>
+          <t>Water while establishing, then only in prolonged dry spells. Do not allow winter waterlogging.</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>Remove old flowering stems at the base with gloves once replacement shoots are clear. Avoid disturbing the crown in cold wet weather.</t>
+          <t>Grow in well-drained soil. Unlike Calluna, winter heath tolerates neutral to mildly alkaline conditions. Trim lightly after flowering without cutting into bare old wood.</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>Compact evergreen mound with yellow-green spring and early-summer flowerheads.</t>
+          <t>Golden evergreen foliage provides year-round colour, with small heath flowers in winter and early spring.</t>
         </is>
       </c>
     </row>
@@ -5563,32 +5563,32 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>Flaming Silver</t>
+          <t>Heather 'Tib'</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>Pieris japonica 'Flaming Silver'</t>
+          <t>Calluna vulgaris 'Tib'</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>Partial shade to sun, sheltered from harsh morning frost.</t>
+          <t>Full sun for compact growth and the best flower display.</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist, especially in dry spells; do not let the rootball dry out.</t>
+          <t>Water while establishing; afterwards it tolerates short dry spells but dislikes waterlogged soil.</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>Ericaceous shrub. Use rainwater where practical and mulch with ericaceous material; prune only lightly after flowering.</t>
+          <t>Needs acidic, well-drained soil. Clip the faded flower spikes lightly in early spring to keep the mound compact, never cutting into bare old wood.</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>Evergreen, cream-edged leaves with red spring growth and cream flowers in spring.</t>
+          <t>Dark evergreen foliage carries double deep-pink flower spikes from July into early autumn.</t>
         </is>
       </c>
     </row>
@@ -5600,32 +5600,32 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Astrantia trio</t>
+          <t>Bell Heather 'Providence' (2 plants)</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>Astrantia major 'Buckland', 'Claret' &amp; 'Star of Love'</t>
+          <t>Daboecia cantabrica 'Providence'</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Sun to light shade.</t>
+          <t>Full sun to partial shade in a position sheltered from cold drying winds.</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>Keep consistently moist during dry weather, particularly while re-establishing.</t>
+          <t>Keep evenly moist while establishing, using rainwater where practical; avoid both drought and waterlogging.</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>Mulch annually with organic matter. Deadhead to prolong flowering and cut back tired stems after flowering.</t>
+          <t>Grow in acidic, humus-rich but freely drained soil. Lightly trim faded stems after flowering without cutting into old wood.</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>Pin-cushion flowers in blush, soft pink and claret shades through summer; foliage dies back in winter.</t>
+          <t>Evergreen mounds with comparatively large, deep rose-red bell flowers through summer and early autumn.</t>
         </is>
       </c>
     </row>
@@ -5637,32 +5637,32 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>Pittosporum 'Tom Thumb'</t>
+          <t>Heather 'Leprechaun'</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>Pittosporum tenuifolium 'Tom Thumb'</t>
+          <t>Calluna vulgaris 'Leprechaun'</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a sheltered position.</t>
+          <t>Full sun for the brightest foliage colour.</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing; later only during prolonged drought. Avoid winter waterlogging.</t>
+          <t>Water while establishing; later, water only during prolonged dry spells and keep the roots well drained.</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>Usually needs little pruning. Remove frost-damaged tips in late spring and protect from cold drying wind.</t>
+          <t>Plant in acidic, freely drained soil. Clip faded flower spikes lightly in spring, avoiding cuts into bare old stems.</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>Lime-green young leaves mature to deep purple, forming a dense rounded evergreen mound.</t>
+          <t>A low evergreen mound with bright lime-gold foliage, pink-tinted new growth and small late-summer flowers.</t>
         </is>
       </c>
     </row>
@@ -5674,32 +5674,32 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Gaura 'Gaudi Red'</t>
+          <t>Heather 'Winter Chocolate'</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>Oenothera lindheimeri 'Florgaured' (Gaudi Red)</t>
+          <t>Calluna vulgaris 'Winter Chocolate'</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Full sun in a warm, sheltered position.</t>
+          <t>Full sun to light partial shade; full sun produces the strongest foliage colour.</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing, then sparingly; sharp winter drainage is essential.</t>
+          <t>Water while establishing; once rooted it tolerates short dry spells but must not sit wet.</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>Deadhead for a longer display. Leave stems over winter and cut back after the worst frosts in spring.</t>
+          <t>Grow in acidic, well-drained soil. Lightly remove old flower spikes in March to prevent the mound becoming woody and leggy.</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>Deep pink-red flowers dance above burgundy-green foliage from summer into autumn.</t>
+          <t>Golden foliage with pink tips in summer turns bronze and chocolate-red in winter; lavender flowers appear August–October.</t>
         </is>
       </c>
     </row>
@@ -5711,32 +5711,32 @@
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>Heather 'Bell's Extra Special'</t>
+          <t>Viola 'Rocky Purple Picotee'</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>Erica carnea 'Bell's Extra Special'</t>
+          <t>Viola cornuta 'Rocky Purple Picotee'</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade; stronger light keeps the foliage richly coloured.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing, then only in prolonged dry spells. Do not allow winter waterlogging.</t>
+          <t>Keep evenly moist while establishing; do not allow the planting pocket to become waterlogged.</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>Grow in well-drained soil. Unlike Calluna, winter heath tolerates neutral to mildly alkaline conditions. Trim lightly after flowering without cutting into bare old wood.</t>
+          <t>Deadhead faded flowers and seed pods regularly to prolong the cool-season display.</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>Golden evergreen foliage provides year-round colour, with small heath flowers in winter and early spring.</t>
+          <t>Purple flowers with pale picotee margins through autumn, winter and spring.</t>
         </is>
       </c>
     </row>
@@ -5748,32 +5748,32 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Heather 'Tib'</t>
+          <t>Ceratostigma</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>Calluna vulgaris 'Tib'</t>
+          <t>Ceratostigma plumbaginoides</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Full sun for compact growth and the best flower display.</t>
+          <t>Full sun to partial shade; flowers and autumn colour are strongest in sun.</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing; afterwards it tolerates short dry spells but dislikes waterlogged soil.</t>
+          <t>Water while establishing, then only in prolonged drought. Prefers soil that drains freely.</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>Needs acidic, well-drained soil. Clip the faded flower spikes lightly in early spring to keep the mound compact, never cutting into bare old wood.</t>
+          <t>Allow room for the rhizomes to spread. Cut old top growth to the ground in spring once new shoots begin to show.</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>Dark evergreen foliage carries double deep-pink flower spikes from July into early autumn.</t>
+          <t>Clear cobalt-blue flowers appear from late summer into autumn as the foliage develops vivid red tints; dormant in winter.</t>
         </is>
       </c>
     </row>
@@ -5785,32 +5785,32 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>Bell Heather 'Providence' (2 plants)</t>
+          <t>Hypericum (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>Daboecia cantabrica 'Providence'</t>
+          <t>Hypericum (cultivar to confirm)</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a position sheltered from cold drying winds.</t>
+          <t>Full sun to partial shade; more sun generally gives stronger flowering.</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist while establishing, using rainwater where practical; avoid both drought and waterlogging.</t>
+          <t>Water while establishing, then during prolonged dry spells only. Avoid persistently waterlogged soil.</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>Grow in acidic, humus-rich but freely drained soil. Lightly trim faded stems after flowering without cutting into old wood.</t>
+          <t>Trim lightly in early spring and remove any weak or damaged stems. Confirm the cultivar from its label, flowers and berries before cultivar-specific pruning.</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>Evergreen mounds with comparatively large, deep rose-red bell flowers through summer and early autumn.</t>
+          <t>A compact shrub grown for golden flowers with prominent stamens and, depending on cultivar, colourful ornamental berries.</t>
         </is>
       </c>
     </row>
@@ -5822,32 +5822,32 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Heather 'Leprechaun'</t>
+          <t>Bluebell Creeper</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>Calluna vulgaris 'Leprechaun'</t>
+          <t>Billardiera heterophylla (syn. Sollya heterophylla)</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>Full sun for the brightest foliage colour.</t>
+          <t>Full sun to partial shade in a warm, sheltered position.</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing; later, water only during prolonged dry spells and keep the roots well drained.</t>
+          <t>Keep evenly moist while establishing, then water during dry spells; avoid waterlogged winter soil.</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>Plant in acidic, freely drained soil. Clip faded flower spikes lightly in spring, avoiding cuts into bare old stems.</t>
+          <t>Tie new shoots into support and trim after flowering to control the twining growth. Protect the root area and young stems during hard frost.</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>A low evergreen mound with bright lime-gold foliage, pink-tinted new growth and small late-summer flowers.</t>
+          <t>A slender evergreen climber with nodding blue bell flowers from summer into autumn, followed by narrow berries when pollinated.</t>
         </is>
       </c>
     </row>
@@ -5859,32 +5859,32 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>Heather 'Winter Chocolate'</t>
+          <t>Hebe 'Rhubarb and Custard'</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Calluna vulgaris 'Winter Chocolate'</t>
+          <t>Veronica 'Tull 302' (Rhubarb and Custard)</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>Full sun to light partial shade; full sun produces the strongest foliage colour.</t>
+          <t>Full sun to partial shade in a warm, sheltered spot.</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing; once rooted it tolerates short dry spells but must not sit wet.</t>
+          <t>Moderate while establishing; drought-tolerant later, but avoid winter waterlogging.</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>Grow in acidic, well-drained soil. Lightly remove old flower spikes in March to prevent the mound becoming woody and leggy.</t>
+          <t>Lightly trim after flowering to keep its rounded shape and protect from severe frost or cold drying winds.</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>Golden foliage with pink tips in summer turns bronze and chocolate-red in winter; lavender flowers appear August–October.</t>
+          <t>Cream-edged grey-green leaves flush pink and rhubarb-red in cold weather; short purple flower spikes appear in mid- to late summer.</t>
         </is>
       </c>
     </row>
@@ -5896,32 +5896,32 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Viola 'Rocky Purple Picotee'</t>
+          <t>Salvia 'Salgoon Lake Blueberry'</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Viola cornuta 'Rocky Purple Picotee'</t>
+          <t>Salvia 'Tl1016' (Salgoon Lake Blueberry)</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Full sun in a warm, sheltered position.</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist while establishing; do not allow the planting pocket to become waterlogged.</t>
+          <t>Water regularly while establishing; once rooted it has good heat and drought tolerance, provided drainage is sharp.</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>Deadhead faded flowers and seed pods regularly to prolong the cool-season display.</t>
+          <t>Deadhead to prolong flowering. Leave top growth over winter, mulch the crown and cut back after the worst frosts in spring; take cuttings as insurance in colder winters.</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>Purple flowers with pale picotee margins through autumn, winter and spring.</t>
+          <t>Compact upright growth to around 60cm with rich blueberry-purple flowers and near-black calyces from summer into autumn.</t>
         </is>
       </c>
     </row>
@@ -5933,814 +5933,629 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>Ceratostigma</t>
+          <t>Fern 'Jurassic Gold'</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Ceratostigma plumbaginoides</t>
+          <t>Dryopteris wallichiana 'Hollasic' (Jurassic Gold)</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; flowers and autumn colour are strongest in sun.</t>
+          <t>Full shade in a sheltered position.</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing, then only in prolonged drought. Prefers soil that drains freely.</t>
+          <t>Shares the existing sprinkler with location 10. Keep moist but well drained while establishing.</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>Allow room for the rhizomes to spread. Cut old top growth to the ground in spring once new shoots begin to show.</t>
+          <t>Mulch well over moist soil, keeping the crown clear. Remove dead or damaged fronds as needed and protect new croziers from late frost and slugs.</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>Clear cobalt-blue flowers appear from late summer into autumn as the foliage develops vivid red tints; dormant in winter.</t>
+          <t>Rose-tinted young fronds mature through bright gold to green; deciduous to semi-evergreen depending on winter.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 5</t>
+          <t>Front Stone Trough</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Hypericum (cultivar to confirm)</t>
+          <t>Hosta</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Hypericum (cultivar to confirm)</t>
+          <t>Hosta</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade; more sun generally gives stronger flowering.</t>
+          <t>Part to full shade.</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing, then during prolonged dry spells only. Avoid persistently waterlogged soil.</t>
+          <t>Keep moist; never bone-dry in the trough.</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>Trim lightly in early spring and remove any weak or damaged stems. Confirm the cultivar from its label, flowers and berries before cultivar-specific pruning.</t>
+          <t>Watch for slugs/snails. Divide clumps in spring.</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>A compact shrub grown for golden flowers with prominent stamens and, depending on cultivar, colourful ornamental berries.</t>
+          <t>Fresh leaves spring; dies back over winter.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 5</t>
+          <t>Front Box Hedge</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>Bluebell Creeper</t>
+          <t>Wall Cotoneaster (species to confirm)</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Billardiera heterophylla (syn. Sollya heterophylla)</t>
+          <t>Cotoneaster (species to confirm)</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a warm, sheltered position.</t>
+          <t>Sun to part shade.</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist while establishing, then water during dry spells; avoid waterlogged winter soil.</t>
+          <t>Water while establishing; once settled, water only in prolonged dry spells.</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>Tie new shoots into support and trim after flowering to control the twining growth. Protect the root area and young stems during hard frost.</t>
+          <t>Train or lightly prune after flowering to keep growth clear of paths and masonry. Do not use box-blight or box-caterpillar treatments. Confirm the species from flowers, berries and leaf undersides.</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>A slender evergreen climber with nodding blue bell flowers from summer into autumn, followed by narrow berries when pollinated.</t>
+          <t>Small leaves on herringbone stems; flowers in late spring or summer followed by red berries. Evergreen or semi-evergreen depending on species and winter.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 5</t>
+          <t>Front Pots</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Hebe 'Rhubarb and Custard'</t>
+          <t>Mixed Pot</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>Veronica 'Tull 302' (Rhubarb and Custard)</t>
+          <t>Mixed seasonal planting — contents to confirm</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>Full sun to partial shade in a warm, sheltered spot.</t>
+          <t>Bright outdoor position; confirm the needs of each constituent plant when identified.</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>Moderate while establishing; drought-tolerant later, but avoid winter waterlogging.</t>
+          <t>Check the compost frequently in warm or windy weather; supplied by an adjustable sprinkler.</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>Lightly trim after flowering to keep its rounded shape and protect from severe frost or cold drying winds.</t>
+          <t>Deadhead finished flowers, keep the drainage holes clear and record the individual plants and cultivars as labels or clearer photographs become available.</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>Cream-edged grey-green leaves flush pink and rhubarb-red in cold weather; short purple flower spikes appear in mid- to late summer.</t>
+          <t>A mixed seasonal container providing varied flower colour; exact contents remain unresolved.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 5</t>
+          <t>Front Pots</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>Salvia 'Salgoon Lake Blueberry'</t>
+          <t>Fuchsia Pot</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Salvia 'Tl1016' (Salgoon Lake Blueberry)</t>
+          <t>Fuchsia cultivars — identities to confirm</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>Full sun in a warm, sheltered position.</t>
+          <t>Bright light or partial shade, protected from the harshest reflected afternoon heat.</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>Water regularly while establishing; once rooted it has good heat and drought tolerance, provided drainage is sharp.</t>
+          <t>Keep the compost evenly moist but freely drained; supplied by an adjustable sprinkler.</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>Deadhead to prolong flowering. Leave top growth over winter, mulch the crown and cut back after the worst frosts in spring; take cuttings as insurance in colder winters.</t>
+          <t>Deadhead for continued flowering, check the sprinkler reaches the compost rather than only the foliage, and confirm whether the plants are hardy before winter.</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>Compact upright growth to around 60cm with rich blueberry-purple flowers and near-black calyces from summer into autumn.</t>
+          <t>Pendant Fuchsia flowers through summer and autumn; exact cultivars and winter hardiness remain unresolved.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Front Bed 5</t>
+          <t>Front Fruit Trees</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Fern 'Jurassic Gold'</t>
+          <t>Apple Tree</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>Dryopteris wallichiana 'Hollasic' (Jurassic Gold)</t>
+          <t>Malus domestica</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>Full shade in a sheltered position.</t>
+          <t>Full sun.</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>Shares the existing sprinkler with location 10. Keep moist but well drained while establishing.</t>
+          <t>Water well in dry spells while fruiting.</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>Mulch well over moist soil, keeping the crown clear. Remove dead or damaged fronds as needed and protect new croziers from late frost and slugs.</t>
+          <t>Winter prune for shape and airflow; thin fruit in June if heavy.</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>Rose-tinted young fronds mature through bright gold to green; deciduous to semi-evergreen depending on winter.</t>
+          <t>Blossom April–May; fruit late summer–autumn.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Front Stone Trough</t>
+          <t>Front Fruit Trees</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>Hosta</t>
+          <t>Damson Tree</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>Hosta</t>
+          <t>Prunus domestica subsp. insititia (cultivar to confirm)</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>Part to full shade.</t>
+          <t>Full sun for reliable blossom and fruit ripening.</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>Keep moist; never bone-dry in the trough.</t>
+          <t>Water deeply during prolonged dry spells, especially from fruit set to harvest.</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>Watch for slugs/snails. Divide clumps in spring.</t>
+          <t>Prune only in dry summer weather to reduce silver-leaf and canker risk; remove suckers from below the graft.</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>Fresh leaves spring; dies back over winter.</t>
+          <t>White spring blossom followed by blue-black damsons in late summer or early autumn.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Front Box Hedge</t>
+          <t>Front Gate Tree</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>Wall Cotoneaster (species to confirm)</t>
+          <t>Weeping Crab Apple (cultivar to confirm)</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>Cotoneaster (species to confirm)</t>
+          <t>Malus (weeping cultivar; 'Red Jade' is a best-fit possibility)</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>Sun to part shade.</t>
+          <t>Full sun for the best blossom, fruit colour and balanced growth.</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>Water while establishing; once settled, water only in prolonged dry spells.</t>
+          <t>Water deeply during prolonged drought, particularly while establishing and while fruit is swelling.</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>Train or lightly prune after flowering to keep growth clear of paths and masonry. Do not use box-blight or box-caterpillar treatments. Confirm the species from flowers, berries and leaf undersides.</t>
+          <t>Remove dead, damaged and crossing wood in winter, preserving the natural weeping framework. Record blossom and ripe-fruit details before naming the cultivar.</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>Small leaves on herringbone stems; flowers in late spring or summer followed by red berries. Evergreen or semi-evergreen depending on species and winter.</t>
+          <t>Spring blossom followed by small ornamental crab apples that can persist into autumn and winter.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Front Pots</t>
+          <t>House · Hallway · Kentia Palm</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>Mixed Pot</t>
+          <t>Kentia Palm — assumed</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>Mixed seasonal planting — contents to confirm</t>
+          <t>Howea forsteriana</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>Bright outdoor position; confirm the needs of each constituent plant when identified.</t>
+          <t>Bright indirect light; protect the fronds from strong direct sun.</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>Check the compost frequently in warm or windy weather; supplied by an adjustable sprinkler.</t>
+          <t>Check the upper few centimetres of compost before watering, then drain fully and empty the white cachepot.</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>Deadhead finished flowers, keep the drainage holes clear and record the individual plants and cultivars as labels or clearer photographs become available.</t>
+          <t>Maintain moderate humidity, keep away from cold draughts and radiators, and feed monthly during active spring and summer growth.</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>A mixed seasonal container providing varied flower colour; exact contents remain unresolved.</t>
+          <t>Evergreen indoor foliage throughout the year; growth slows as light levels fall in winter.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Front Pots</t>
+          <t>House · Sitting Room · ‘Gioia’ Fern</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Fuchsia Pot</t>
+          <t>Bird’s Nest Fern ‘Gioia’</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>Fuchsia cultivars — identities to confirm</t>
+          <t>Asplenium antiquum ‘Gioia’</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>Bright light or partial shade, protected from the harshest reflected afternoon heat.</t>
+          <t>Bright, indirect light; protect the fronds from direct sun through the glass.</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>Keep the compost evenly moist but freely drained; supplied by an adjustable sprinkler.</t>
+          <t>Keep compost lightly moist but never saturated; water around the pot edge rather than into the centre rosette.</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>Deadhead for continued flowering, check the sprinkler reaches the compost rather than only the foliage, and confirm whether the plants are hardy before winter.</t>
+          <t>Give it steady warmth and higher humidity, removing only damaged fronds at the base.</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>Pendant Fuchsia flowers through summer and autumn; exact cultivars and winter hardiness remain unresolved.</t>
+          <t>Evergreen indoor foliage throughout the year; growth slows in lower winter light.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Front Fruit Trees</t>
+          <t>House · Hallway · Staghorn Fern</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>Apple Tree</t>
+          <t>Staghorn Fern</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>Malus domestica</t>
+          <t>Platycerium bifurcatum</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>Full sun.</t>
+          <t>Bright, indirect light; avoid harsh midday sun and cold draughts.</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>Water well in dry spells while fruiting.</t>
+          <t>Check the growing medium before watering and let excess water drain completely; never keep the base wet.</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>Winter prune for shape and airflow; thin fruit in June if heavy.</t>
+          <t>Maintain moderate humidity and keep the fern clear of direct radiator heat. Leave the brown papery shield fronds in place.</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>Blossom April–May; fruit late summer–autumn.</t>
+          <t>Evergreen antler-like fronds are the display throughout the year; growth is slower in winter.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Front Fruit Trees</t>
+          <t>Skimmia Pot</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Damson Tree</t>
+          <t>Skimmia 'Cleopatra'</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Prunus domestica subsp. insititia (cultivar to confirm)</t>
+          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>Full sun for reliable blossom and fruit ripening.</t>
+          <t>Light to full shade, sheltered from harsh sun and drying wind.</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>Water deeply during prolonged dry spells, especially from fruit set to harvest.</t>
+          <t>Keep the shared compost consistently moist but well drained, preferably using rainwater.</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>Prune only in dry summer weather to reduce silver-leaf and canker risk; remove suckers from below the graft.</t>
+          <t>Mulch or top-dress with leaf mould or ericaceous compost. Prune only lightly after flowering and keep ivy stems away from its crown.</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>White spring blossom followed by blue-black damsons in late summer or early autumn.</t>
+          <t>Glossy evergreen foliage, fragrant ivory spring flowers and long-lasting red berries from autumn into winter.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Front Gate Tree</t>
+          <t>Skimmia Pot</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Weeping Crab Apple (cultivar to confirm)</t>
+          <t>Skimmia 'Antarctica'</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Malus (weeping cultivar; 'Red Jade' is a best-fit possibility)</t>
+          <t>Skimmia 'Antarctica'</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>Full sun for the best blossom, fruit colour and balanced growth.</t>
+          <t>Partial to full shade, sheltered from harsh sun and drying wind.</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>Water deeply during prolonged drought, particularly while establishing and while fruit is swelling.</t>
+          <t>Keep compost evenly moist and freely drained; rainwater is preferred where practical.</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>Remove dead, damaged and crossing wood in winter, preserving the natural weeping framework. Record blossom and ripe-fruit details before naming the cultivar.</t>
+          <t>Use ericaceous compost and prune only lightly after flowering. Do not let the root ball dry out while establishing.</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>Spring blossom followed by small ornamental crab apples that can persist into autumn and winter.</t>
+          <t>Glossy evergreen foliage and spring flower buds give year-round structure.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>House · Hallway · Kentia Palm</t>
+          <t>Skimmia Pot</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Kentia Palm — assumed</t>
+          <t>Viola 'Rocky Purple Picotee' (3 plants)</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Howea forsteriana</t>
+          <t>Viola cornuta 'Rocky Purple Picotee'</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>Bright indirect light; protect the fronds from strong direct sun.</t>
+          <t>Sun to partial shade.</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>Check the upper few centimetres of compost before watering, then drain fully and empty the white cachepot.</t>
+          <t>Keep the shared compost evenly moist but well drained.</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>Maintain moderate humidity, keep away from cold draughts and radiators, and feed monthly during active spring and summer growth.</t>
+          <t>Deadhead faded flowers and seed pods regularly to prolong flowering.</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>Evergreen indoor foliage throughout the year; growth slows as light levels fall in winter.</t>
+          <t>Purple flowers with pale picotee margins through the cool season.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>House · Sitting Room · ‘Gioia’ Fern</t>
+          <t>Bed 2/3 Wall Pot</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>Bird’s Nest Fern ‘Gioia’</t>
+          <t>Viburnum 'Lisarose'</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Asplenium antiquum ‘Gioia’</t>
+          <t>Viburnum tinus 'Lisarose'</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>Bright, indirect light; protect the fronds from direct sun through the glass.</t>
+          <t>Sun, partial shade or shade, sheltered from cold drying winds.</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>Keep compost lightly moist but never saturated; water around the pot edge rather than into the centre rosette.</t>
+          <t>Keep evenly moist while establishing; never leave the container waterlogged.</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>Give it steady warmth and higher humidity, removing only damaged fronds at the base.</t>
+          <t>Use humus-rich, well-drained compost. Prune only after flowering if its size needs controlling.</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>Evergreen indoor foliage throughout the year; growth slows in lower winter light.</t>
+          <t>Brick-red winter buds open to pink-and-white flowers, followed by dark blue ornamental berries.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>House · Hallway · Staghorn Fern</t>
+          <t>Bed 2/3 Wall Pot</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Staghorn Fern</t>
+          <t>Vinca minor 'Illumination'</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Platycerium bifurcatum</t>
+          <t>Vinca minor 'Illumination'</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>Bright, indirect light; avoid harsh midday sun and cold draughts.</t>
+          <t>Sun to shade; foliage colours best in bright indirect light or partial shade.</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>Check the growing medium before watering and let excess water drain completely; never keep the base wet.</t>
+          <t>Moderate. Let the surface dry slightly without allowing the pot to dry completely.</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>Maintain moderate humidity and keep the fern clear of direct radiator heat. Leave the brown papery shield fronds in place.</t>
+          <t>Trim trailing stems to shape and keep drainage holes clear. Do not plant into open ground without a spread plan.</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>Evergreen antler-like fronds are the display throughout the year; growth is slower in winter.</t>
+          <t>Golden evergreen foliage with narrow green margins and violet-blue flowers from spring into autumn.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>Skimmia Pot</t>
+          <t>Viburnum Pot</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>Skimmia 'Cleopatra'</t>
+          <t>Viburnum tinus Spirit</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
+          <t>Viburnum tinus 'Anvi' (Spirit)</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>Light to full shade, sheltered from harsh sun and drying wind.</t>
+          <t>Sun or partial shade, with shelter from cold drying winds.</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>Keep the shared compost consistently moist but well drained, preferably using rainwater.</t>
+          <t>Keep evenly moist but well drained while establishing; check the pot through dry and windy weather.</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>Mulch or top-dress with leaf mould or ericaceous compost. Prune only lightly after flowering and keep ivy stems away from its crown.</t>
+          <t>Prune only after flowering if needed. Refresh the top compost in spring and protect the container during prolonged severe cold.</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>Glossy evergreen foliage, fragrant ivory spring flowers and long-lasting red berries from autumn into winter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="2" t="inlineStr">
-        <is>
-          <t>Skimmia Pot</t>
-        </is>
-      </c>
-      <c r="B166" s="2" t="inlineStr">
-        <is>
-          <t>Skimmia 'Antarctica'</t>
-        </is>
-      </c>
-      <c r="C166" s="2" t="inlineStr">
-        <is>
-          <t>Skimmia 'Antarctica'</t>
-        </is>
-      </c>
-      <c r="D166" s="2" t="inlineStr">
-        <is>
-          <t>Partial to full shade, sheltered from harsh sun and drying wind.</t>
-        </is>
-      </c>
-      <c r="E166" s="2" t="inlineStr">
-        <is>
-          <t>Keep compost evenly moist and freely drained; rainwater is preferred where practical.</t>
-        </is>
-      </c>
-      <c r="F166" s="2" t="inlineStr">
-        <is>
-          <t>Use ericaceous compost and prune only lightly after flowering. Do not let the root ball dry out while establishing.</t>
-        </is>
-      </c>
-      <c r="G166" s="2" t="inlineStr">
-        <is>
-          <t>Glossy evergreen foliage and spring flower buds give year-round structure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="2" t="inlineStr">
-        <is>
-          <t>Skimmia Pot</t>
-        </is>
-      </c>
-      <c r="B167" s="2" t="inlineStr">
-        <is>
-          <t>Viola 'Rocky Purple Picotee' (3 plants)</t>
-        </is>
-      </c>
-      <c r="C167" s="2" t="inlineStr">
-        <is>
-          <t>Viola cornuta 'Rocky Purple Picotee'</t>
-        </is>
-      </c>
-      <c r="D167" s="2" t="inlineStr">
-        <is>
-          <t>Sun to partial shade.</t>
-        </is>
-      </c>
-      <c r="E167" s="2" t="inlineStr">
-        <is>
-          <t>Keep the shared compost evenly moist but well drained.</t>
-        </is>
-      </c>
-      <c r="F167" s="2" t="inlineStr">
-        <is>
-          <t>Deadhead faded flowers and seed pods regularly to prolong flowering.</t>
-        </is>
-      </c>
-      <c r="G167" s="2" t="inlineStr">
-        <is>
-          <t>Purple flowers with pale picotee margins through the cool season.</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="2" t="inlineStr">
-        <is>
-          <t>Bed 2/3 Wall Pot</t>
-        </is>
-      </c>
-      <c r="B168" s="2" t="inlineStr">
-        <is>
-          <t>Viburnum 'Lisarose'</t>
-        </is>
-      </c>
-      <c r="C168" s="2" t="inlineStr">
-        <is>
-          <t>Viburnum tinus 'Lisarose'</t>
-        </is>
-      </c>
-      <c r="D168" s="2" t="inlineStr">
-        <is>
-          <t>Sun, partial shade or shade, sheltered from cold drying winds.</t>
-        </is>
-      </c>
-      <c r="E168" s="2" t="inlineStr">
-        <is>
-          <t>Keep evenly moist while establishing; never leave the container waterlogged.</t>
-        </is>
-      </c>
-      <c r="F168" s="2" t="inlineStr">
-        <is>
-          <t>Use humus-rich, well-drained compost. Prune only after flowering if its size needs controlling.</t>
-        </is>
-      </c>
-      <c r="G168" s="2" t="inlineStr">
-        <is>
-          <t>Brick-red winter buds open to pink-and-white flowers, followed by dark blue ornamental berries.</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="2" t="inlineStr">
-        <is>
-          <t>Bed 2/3 Wall Pot</t>
-        </is>
-      </c>
-      <c r="B169" s="2" t="inlineStr">
-        <is>
-          <t>Vinca minor 'Illumination'</t>
-        </is>
-      </c>
-      <c r="C169" s="2" t="inlineStr">
-        <is>
-          <t>Vinca minor 'Illumination'</t>
-        </is>
-      </c>
-      <c r="D169" s="2" t="inlineStr">
-        <is>
-          <t>Sun to shade; foliage colours best in bright indirect light or partial shade.</t>
-        </is>
-      </c>
-      <c r="E169" s="2" t="inlineStr">
-        <is>
-          <t>Moderate. Let the surface dry slightly without allowing the pot to dry completely.</t>
-        </is>
-      </c>
-      <c r="F169" s="2" t="inlineStr">
-        <is>
-          <t>Trim trailing stems to shape and keep drainage holes clear. Do not plant into open ground without a spread plan.</t>
-        </is>
-      </c>
-      <c r="G169" s="2" t="inlineStr">
-        <is>
-          <t>Golden evergreen foliage with narrow green margins and violet-blue flowers from spring into autumn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="2" t="inlineStr">
-        <is>
-          <t>Viburnum Pot</t>
-        </is>
-      </c>
-      <c r="B170" s="2" t="inlineStr">
-        <is>
-          <t>Viburnum tinus Spirit</t>
-        </is>
-      </c>
-      <c r="C170" s="2" t="inlineStr">
-        <is>
-          <t>Viburnum tinus 'Anvi' (Spirit)</t>
-        </is>
-      </c>
-      <c r="D170" s="2" t="inlineStr">
-        <is>
-          <t>Sun or partial shade, with shelter from cold drying winds.</t>
-        </is>
-      </c>
-      <c r="E170" s="2" t="inlineStr">
-        <is>
-          <t>Keep evenly moist but well drained while establishing; check the pot through dry and windy weather.</t>
-        </is>
-      </c>
-      <c r="F170" s="2" t="inlineStr">
-        <is>
-          <t>Prune only after flowering if needed. Refresh the top compost in spring and protect the container during prolonged severe cold.</t>
-        </is>
-      </c>
-      <c r="G170" s="2" t="inlineStr">
-        <is>
           <t>Pink buds open to lightly fragrant creamy-white flowers from late winter into spring, followed by blue-black ornamental berries.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G170"/>
+  <autoFilter ref="A1:G165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Nicola's mixed houseplant pot and move Gioia
</commit_message>
<xml_diff>
--- a/Oak_Lodge_Garden_Plant_Guide.xlsx
+++ b/Oak_Lodge_Garden_Plant_Guide.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plant Guide" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$G$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plant Guide'!$A$1:$G$168</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Plant Guide'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G165"/>
+  <dimension ref="A1:G168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6261,7 +6261,7 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>House · Sitting Room · ‘Gioia’ Fern</t>
+          <t>House · Kitchen / Dining · ‘Gioia’ Fern</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -6335,227 +6335,338 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Skimmia Pot</t>
+          <t>House · Sitting Room · Shared Pot · Spider Plant</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Skimmia 'Cleopatra'</t>
+          <t>Spider Plant ‘Vittatum’ — assumed</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
+          <t>Chlorophytum comosum ‘Vittatum’</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>Light to full shade, sheltered from harsh sun and drying wind.</t>
+          <t>Bright indirect light is ideal; it tolerates lower light but direct hot sun can scorch the striped leaves.</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>Keep the shared compost consistently moist but well drained, preferably using rainwater.</t>
+          <t>Allow the compost surface to begin drying, then water thoroughly and let the shared container drain fully.</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>Mulch or top-dress with leaf mould or ericaceous compost. Prune only lightly after flowering and keep ivy stems away from its crown.</t>
+          <t>Trim only spent stems or badly damaged leaves, feed lightly during active growth and root the hanging plantlets if wanted.</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>Glossy evergreen foliage, fragrant ivory spring flowers and long-lasting red berries from autumn into winter.</t>
+          <t>Evergreen striped foliage and hanging plantlets are the year-round display; growth slows in winter.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Skimmia Pot</t>
+          <t>House · Sitting Room · Shared Pot · Parlour Palm</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Skimmia 'Antarctica'</t>
+          <t>Parlour Palm — assumed</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Skimmia 'Antarctica'</t>
+          <t>Chamaedorea elegans</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>Partial to full shade, sheltered from harsh sun and drying wind.</t>
+          <t>Bright indirect light or light shade; protect the fine leaflets from strong direct sun.</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>Keep compost evenly moist and freely drained; rainwater is preferred where practical.</t>
+          <t>Check below the surface before watering; keep lightly moist in growth but never leave the shared planter waterlogged.</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>Use ericaceous compost and prune only lightly after flowering. Do not let the root ball dry out while establishing.</t>
+          <t>Keep warm, remove only fully brown fronds at the base and feed monthly at low strength in spring and summer.</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>Glossy evergreen foliage and spring flower buds give year-round structure.</t>
+          <t>Evergreen fine-textured fronds provide the display throughout the year; growth is slowest in winter.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Skimmia Pot</t>
+          <t>House · Sitting Room · Shared Pot · Arrowhead Vine</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Viola 'Rocky Purple Picotee' (3 plants)</t>
+          <t>Arrowhead Vine — assumed</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Viola cornuta 'Rocky Purple Picotee'</t>
+          <t>Syngonium podophyllum</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>Sun to partial shade.</t>
+          <t>Bright indirect light; keep the leaves out of strong direct sun through the glass.</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>Keep the shared compost evenly moist but well drained.</t>
+          <t>Keep lightly moist during active growth, allowing the surface to begin drying; water more sparingly in winter.</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>Deadhead faded flowers and seed pods regularly to prolong flowering.</t>
+          <t>Guide or trim lengthening stems in spring, feed during active growth and wear gloves if pruning because the sap is irritating.</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>Purple flowers with pale picotee margins through the cool season.</t>
+          <t>Evergreen juvenile arrow-shaped leaves become more divided as stems mature; indoor flowering is uncommon.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>Bed 2/3 Wall Pot</t>
+          <t>Skimmia Pot</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>Viburnum 'Lisarose'</t>
+          <t>Skimmia 'Cleopatra'</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Viburnum tinus 'Lisarose'</t>
+          <t>Skimmia japonica 'Snep24' (Cleopatra)</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>Sun, partial shade or shade, sheltered from cold drying winds.</t>
+          <t>Light to full shade, sheltered from harsh sun and drying wind.</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>Keep evenly moist while establishing; never leave the container waterlogged.</t>
+          <t>Keep the shared compost consistently moist but well drained, preferably using rainwater.</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>Use humus-rich, well-drained compost. Prune only after flowering if its size needs controlling.</t>
+          <t>Mulch or top-dress with leaf mould or ericaceous compost. Prune only lightly after flowering and keep ivy stems away from its crown.</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>Brick-red winter buds open to pink-and-white flowers, followed by dark blue ornamental berries.</t>
+          <t>Glossy evergreen foliage, fragrant ivory spring flowers and long-lasting red berries from autumn into winter.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Bed 2/3 Wall Pot</t>
+          <t>Skimmia Pot</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Vinca minor 'Illumination'</t>
+          <t>Skimmia 'Antarctica'</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Vinca minor 'Illumination'</t>
+          <t>Skimmia 'Antarctica'</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>Sun to shade; foliage colours best in bright indirect light or partial shade.</t>
+          <t>Partial to full shade, sheltered from harsh sun and drying wind.</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>Moderate. Let the surface dry slightly without allowing the pot to dry completely.</t>
+          <t>Keep compost evenly moist and freely drained; rainwater is preferred where practical.</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>Trim trailing stems to shape and keep drainage holes clear. Do not plant into open ground without a spread plan.</t>
+          <t>Use ericaceous compost and prune only lightly after flowering. Do not let the root ball dry out while establishing.</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>Golden evergreen foliage with narrow green margins and violet-blue flowers from spring into autumn.</t>
+          <t>Glossy evergreen foliage and spring flower buds give year-round structure.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
+          <t>Skimmia Pot</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Viola 'Rocky Purple Picotee' (3 plants)</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Viola cornuta 'Rocky Purple Picotee'</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>Sun to partial shade.</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>Keep the shared compost evenly moist but well drained.</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>Deadhead faded flowers and seed pods regularly to prolong flowering.</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>Purple flowers with pale picotee margins through the cool season.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>Bed 2/3 Wall Pot</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Viburnum 'Lisarose'</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Viburnum tinus 'Lisarose'</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>Sun, partial shade or shade, sheltered from cold drying winds.</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>Keep evenly moist while establishing; never leave the container waterlogged.</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>Use humus-rich, well-drained compost. Prune only after flowering if its size needs controlling.</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>Brick-red winter buds open to pink-and-white flowers, followed by dark blue ornamental berries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>Bed 2/3 Wall Pot</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>Vinca minor 'Illumination'</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Vinca minor 'Illumination'</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>Sun to shade; foliage colours best in bright indirect light or partial shade.</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>Moderate. Let the surface dry slightly without allowing the pot to dry completely.</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>Trim trailing stems to shape and keep drainage holes clear. Do not plant into open ground without a spread plan.</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>Golden evergreen foliage with narrow green margins and violet-blue flowers from spring into autumn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
           <t>Viburnum Pot</t>
         </is>
       </c>
-      <c r="B165" s="2" t="inlineStr">
+      <c r="B168" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus Spirit</t>
         </is>
       </c>
-      <c r="C165" s="2" t="inlineStr">
+      <c r="C168" s="2" t="inlineStr">
         <is>
           <t>Viburnum tinus 'Anvi' (Spirit)</t>
         </is>
       </c>
-      <c r="D165" s="2" t="inlineStr">
+      <c r="D168" s="2" t="inlineStr">
         <is>
           <t>Sun or partial shade, with shelter from cold drying winds.</t>
         </is>
       </c>
-      <c r="E165" s="2" t="inlineStr">
+      <c r="E168" s="2" t="inlineStr">
         <is>
           <t>Keep evenly moist but well drained while establishing; check the pot through dry and windy weather.</t>
         </is>
       </c>
-      <c r="F165" s="2" t="inlineStr">
+      <c r="F168" s="2" t="inlineStr">
         <is>
           <t>Prune only after flowering if needed. Refresh the top compost in spring and protect the container during prolonged severe cold.</t>
         </is>
       </c>
-      <c r="G165" s="2" t="inlineStr">
+      <c r="G168" s="2" t="inlineStr">
         <is>
           <t>Pink buds open to lightly fragrant creamy-white flowers from late winter into spring, followed by blue-black ornamental berries.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G165"/>
+  <autoFilter ref="A1:G168"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>